<commit_message>
Move job post link next to role in last-week Excel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MVEsxJLMD4NEiYeySLLsQo
</commit_message>
<xml_diff>
--- a/linkedin_jobs/output/java_selenium_hyderabad_last_week.xlsx
+++ b/linkedin_jobs/output/java_selenium_hyderabad_last_week.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Last 7 days" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Last 7 days'!$A$1:$I$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Last 7 days'!$A$1:$H$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -59,10 +59,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,18 +432,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="80" customWidth="1" min="9" max="9"/>
+    <col width="80" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -451,19 +453,19 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Job Post Link</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Seniority Level</t>
@@ -480,11 +482,6 @@
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Url</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
@@ -496,21 +493,21 @@
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Automation test engineer</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/automation-test-engineer-at-infosys-4472383558</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>Infosys</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -526,12 +523,7 @@
           <t>49 applicants</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/automation-test-engineer-at-infosys-4472383558</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Technology-&gt;Automated Testing-&gt;Selenium-Java Design, develop, and maintain scalable automation test frameworks using Java and Selenium WebDriver. Create, execute, and maintain automated test scripts for web applications. Perform functional, regression, integration, and smoke testing. Analyze test results, identify defects, and collaborate with development teams for issue resolution. Develop and maintain test plans, test cases, and test data. Integrate automation suites with CI/CD pipelines using Jenkins, Azure DevOps, or GitLab. Perform API testing using tools such as Postman or Rest Assured. Participate in Agile ceremonies including sprint planning, daily stand-ups, and retrospectives. Generate test execution reports and quality metrics. Ensure adherence to software testing best practices and quality standards.</t>
         </is>
@@ -543,21 +535,21 @@
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Automation Test Engineer</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/automation-test-engineer-at-luxoft-4474111385</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>Luxoft</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>Associate</t>
@@ -573,12 +565,7 @@
           <t>174 applicants</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/automation-test-engineer-at-luxoft-4474111385</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Project Description: Join a high-performing Agile pod as a Mid-Level QA Engineer, supporting both automated and manual testing of integration endpoints. You'll work closely with senior engineers to enhance test coverage, improve quality, and leverage AI-assisted testing tools to accelerate development, defect detection, and testing efficiency. Responsibilities: Write and maintain automated test scripts for REST APIs and integration workflows Execute manual tests, identify defects, and support root cause analysis Work closely with developers to validate functionality and ensure quality across features Participate in Agile ceremonies and contribute to sprint reviews and planning Assist in maintaining test data and improving test coverage Leverage AI-assisted tools to support test case creation, debugging, and test data generation Mandatory Skills Description: 2-4 years of QA experience in Agile environments Testing &amp; Automation: Experience with test automation tools (e.g., Selenium, Postman) Good understanding of API and integration testing concepts Familiarity with writing and executing automated and manual test cases Understanding of various test types and creating test plans for releases Python Skill set for automation testing Technical Skills: Familiarity with basic scripting or Java-based test frameworks Understanding of REST APIs and JSON-based data exchange DevOps &amp; Tooling: Exposure to CI/CD tools (e.g., GitLab, Jenkins) Familiarity with version control systems AI-Assisted Testing: Exposure to AI-assisted coding and testing tools (e.g., GitLab Copilot, IDE-based copilots) Familiarity with using generative AI for test case suggestions, script generation, debugging, and documentation Eagerness to adopt AI tools to improve efficiency, learning, and test quality Collaboration: Strong collaboration and communication skills Nice-to-Have Skills Description: Ability to work effectively in Agile teams and learn from senior engineers</t>
         </is>
@@ -590,21 +577,21 @@
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Manager, Software Development &amp; Engineering</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/manager-software-development-engineering-at-charles-schwab-india-4474129345</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>Charles Schwab India</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -620,12 +607,7 @@
           <t>Be among the first 25 applicants</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/manager-software-development-engineering-at-charles-schwab-india-4474129345</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Your opportunity Schwab Description At Charles Schwab, our purpose is simple: we championclient’sgoals with passion and integrity. Guided by honesty, mutualrespectand a commitment to doingwhat’sright, we bring innovation, education, and service together to help shape financial futures. Our people are the foundation of our success - they approach their work with curiosity and collaboration, coming together to create solutions that make a meaningful impact for clients and communities. As we expand into India, we are bringing this same culture of inclusion, learning, and opportunity to new talent. Joining us means becoming part of a global team where your work matters and your future can take shape. Schwab India Description Our Hyderabad location is central to Schwab’s growth, bringing together talented people and technology to drive innovation,scaleand efficiency. Here, you will work alongside teams who create solutions that support millions of clients every day. The work you do is more than daily operations -it’sa chance to experiment, learn, and build within avalues-driven, supportive environment. This is a unique opportunity to be part of our early growth phase and shape something new, backed by the stability and strength of a Fortune 500 company. Your impact begins on day one, and your contributions will help define our future in the region. Role Description We’reseeking a Senior QA Engineer to lead program-level end-to-end test planning and execution across complex, distributed systems. This role owns QA strategy and delivery for high-impact initiatives,establishesand scales test automation, and drives non-production environment and test data readiness so teams can release confidently and on time. What you have Key Responsibilities Define and govern the program-level E2E testing approach, including scope, entry/exit criteria, risk-based design, orchestration, reporting, and remediation. Lead multi-application and partner integrations,coordinatingdependencies, cross-domain scenarios, and releasesign-offs. Establish dashboards and operating rhythms for preparation, execution, triage, and RCA. Build reliable and maintainable regression, smoke, and feature validation test suites. Embed automation in sprint workflows and mentor SDETs and QA engineers. Own readiness of non-production environments and test data for E2E scenarios. Drive triage and escalation using TEMS workflows to unblock testing. Partner with Product Owners, Scrum Masters, and engineering leads tocommunicatestatus, risks, and decisions. Required Qualifications 8 - 10+ years in Software QA Engineering with a strong record of delivering quality in complex programs. 7+ years leading E2E test programs across multiple applications and partners. 6+ years hands-on test automation for UI/API/service testing, including framework design and CI/CD integration. Experience defining and executing multi-year QA roadmaps and program-level test strategies. Proven collaboration with business and technology stakeholders with clear communication of risks, decisions, andsign-offs. Experience leading E2E QA and UAT coordinators, test environments, and test data pipelines. Ability to provide QA sign-off and RCA recommendations forimplementations. Experience ensuring risk-based testing, agreed test approaches, high-quality deliverables,accuratereporting, and active risk/issue management. Ability to generate innovative QA solutions, improve audit compliance, organize/prioritize requirements, andoptimizesoftware testing and verification. Preferred Qualifications ExpertiseinSAFeand Scrum. Test Automation and Process Optimization framework design and implementation. Ability to lead and inspire teams through complex and changing circumstances. Experience with GitHub, Bitbucket, Bamboo, Splunk, Postman, andMabl. Hands-on Java/Javascript/Selenium or BDD-driven automation frameworks. Deep understanding of exploratory testing practices. Working knowledge of JIRA/MTM, Zephyr/HPQ, service virtualization, test data management, CI/CD, Lean DevOps, and financial/move money/payment/trading domain experience. What’s in it for you At Schwab India, you’re empowered to shape your future. We support your growth through meaningful work, continuous learning, and a culture rooted in trust and collaboration – so you can build the skills to make a lasting impact. Our benefits are designed to care for your wellbeing, your family, and your long-term financial security. Our Base Benefits, Wellbeing, And Total Rewards Include Competitive compensation and retirement programs including Employee Provident Fund (EPF), Gratuity, and optional National Pension System (NPS) contributions Robust Paid Time Off, including annual/privilege leave, sick and casual leave, public holidays, maternity/paternity leave, and more Comprehensive medical insurance with Outpatient Department (OPD) services, including vaccination, pharmacy, dental, and vision coverage Annual reimbursement for health check-ups and mental health support through our Employee Assistance Program (EAP) Childcare (creche) reimbursement for eligible employees Transportation and meal benefits that support your day-to-day work Group life, personal accident, and critical illness insurance Apply</t>
         </is>
@@ -637,21 +619,21 @@
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Automation Test lead</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/automation-test-lead-at-infosys-4472379642</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>Infosys</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -667,12 +649,7 @@
           <t>Be among the first 25 applicants</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/automation-test-lead-at-infosys-4472379642</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Technology-&gt;Automated Testing-&gt;Selenium-Java Design, develop, and maintain scalable automation test frameworks using Java and Selenium WebDriver. Create, execute, and maintain automated test scripts for web applications. Perform functional, regression, integration, and smoke testing. Analyze test results, identify defects, and collaborate with development teams for issue resolution. Develop and maintain test plans, test cases, and test data. Integrate automation suites with CI/CD pipelines using Jenkins, Azure DevOps, or GitLab. Perform API testing using tools such as Postman or Rest Assured. Participate in Agile ceremonies including sprint planning, daily stand-ups, and retrospectives. Generate test execution reports and quality metrics. Ensure adherence to software testing best practices and quality standards.</t>
         </is>
@@ -684,21 +661,21 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Senior Testing Lead - Automation, Performance, Security &amp; Functional QA</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/senior-testing-lead-automation-performance-security-functional-qa-at-petadata-4473946023</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
         <is>
           <t>PETADATA</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>Mid-Senior level</t>
@@ -714,12 +691,7 @@
           <t>99 applicants</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/senior-testing-lead-automation-performance-security-functional-qa-at-petadata-4473946023</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Position: Senior Testing Lead - Automation, Performance, Security &amp; Functional QA Location: Hyderabad ( 8 PM to 5 AM IST) Work Type: Full-Time/Onsite Experience: 8+ Years PETADATA is looking for a highly experienced Senior Testing Lead with 8+ years of experience to own the overall quality strategy, build and scale test automation, and lead functional, performance, security, API, and data-validation testing for a data migration platform operating across cloud and on-premise environments. Roles &amp; Responsibilities Quality Strategy &amp; Leadership Own and define the overall QA and testing strategy across functional, automation, performance, security, and data-integrity testing. Establish quality gates, release criteria, testing standards, metrics, and reporting. Identify and prioritize testing efforts based on business and technical risk, especially data-correctness risks. Build and manage the quality function with minimal supervision. Mentor developers and QA engineers and promote a quality-first engineering culture. Partner closely with Engineering, DevOps, Architecture, Security, and Implementation teams. Test Automation Design and build test automation frameworks from scratch. Develop automated UI, API, integration, and regression testing solutions. Use tools such as Playwright, Cypress, Selenium, and REST/API automation frameworks. Integrate automated testing into CI/CD pipelines. Build scalable regression suites that improve release velocity and confidence. Use programming languages such as Python, JavaScript/TypeScript, or Java for automation. Functional &amp; Migration Testing Own end-to-end functional testing across supported CRM platforms and migration scenarios. Test standard and custom objects, relationships, transformations, mappings, and edge cases. Design test scenarios based on real-world customer data migration use cases. Validate migration correctness from source to destination. Test multi-tenant behavior, configuration, and tenant data isolation. Identify defects and ensure issues are properly investigated, resolved, and prevented from recurring. Data Validation &amp; Integrity Build automated source-to-target data validation frameworks. Validate: Record counts Field-level accuracy Data mappings Relationships and associations Transformations Deduplication Overall data integrity Use SQL and programmatic validation techniques to verify migration results. Ensure migrated customer data remains complete, accurate, and consistent. Performance Testing Design and execute load, stress, scalability, and performance testing. Test large data volumes and high numbers of concurrent migrations. Establish performance baselines, benchmarks, and SLAs. Identify performance bottlenecks and work with Engineering and Architecture teams to resolve them. Use tools such as k6, JMeter, Gatling, or Locust. Integrate appropriate performance testing into the CI/CD pipeline. Security Testing Perform and coordinate security testing across the application and platform. Test tenant isolation and ensure no cross-tenant data access is possible. Validate authentication and authorization controls. Perform input validation and abuse-case testing. Integrate SAST, DAST, and vulnerability scanning into CI/CD. Coordinate penetration testing with internal security teams and external security vendors. Support security and compliance requirements such as SOC 2 and ISO 27001 through appropriate testing evidence. Technical Quality &amp; Delivery Ensure software is secure, scalable, reliable, and production-ready. Establish automated quality checks throughout the development lifecycle. Collaborate with developers to identify defects early. Review testing approaches and improve overall engineering quality. Support both cloud and on-premise deployments. Help establish reliable test environments using cloud, containers, and infrastructure automation. Note: Should be highly self-directed, comfortable building the QA function from the ground up, and able to work effectively with distributed engineering teams across required time zones. Note: Should be able to work independently and work in USA time zones Required Skills 8+ years of professional QA / Test Engineering experience. Strong experience leading QA strategy and quality engineering for software products. Strong hands-on experience building test automation frameworks from scratch. Proficiency with Playwright, Cypress, and/or Selenium. Strong API and REST testing experience. Strong programming experience with Python, JavaScript/TypeScript, or Java. Hands-on experience integrating automated testing into CI/CD pipelines. Experience with functional, integration, regression, and end-to-end testing. Strong experience with performance/load testing using JMeter, k6, Gatling, Locust, or similar tools. Working knowledge of security testing, including OWASP, authentication, authorization, tenant isolation, SAST, DAST, and vulnerability scanning. Strong SQL and data-validation experience. Experience validating source-to-target data integrity across multiple systems. Strong understanding of data migration, ETL, integration, or data-intensive applications. Experience testing multi-tenant SaaS applications. Experience with cloud platforms such as AWS, Azure, or GCP. Experience with on-premise/customer-deployed software is preferred. Experience with Salesforce, HubSpot, Zoho, or similar CRM platforms is a plus. Familiarity with Docker, containers, and IaC is a plus. Exposure to chaos/resilience testing or contract testing is a plus. Experience supporting SOC 2 / ISO 27001 or other compliance audits is preferred. Strong problem-solving, communication, leadership, ownership, and decision-making skills. Ability to independently establish testing processes, frameworks, quality standards, and release criteria. Education Bachelor s degree in Computer Science, Information Technology, Engineering, or a related field is preferred. Candidates must attend phone/video calls and in-person interviews as required. After selection, candidates will undergo background checks on Education and Experience. Please email your resume to pavanm@petadata.ai After carefully reviewing your experience and skills, one of our HR team members will contact you about the next steps.</t>
         </is>
@@ -731,21 +703,21 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Quality Assurance Engineer - Automation Testing</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/quality-assurance-engineer-automation-testing-at-scoutit-4471998627</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>Scoutit</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>Mid-Senior level</t>
@@ -761,12 +733,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/quality-assurance-engineer-automation-testing-at-scoutit-4471998627</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>We're looking for Quality Assurance Engineers - Automation Testing ! Responsibilities: Design and develop automated test scripts using tools like Selenium, TestNG, or similar frameworks. Execute automated test scripts and analyze results to ensure software quality. Collaborate with development teams to understand project requirements and provide feedback on testing processes. Maintain and update existing automated test cases as necessary to reflect changes in application functionality. Report and track defects found during testing and verify fixes in subsequent builds. Be a team player and work across teams. Qualifications: Proficiency in software testing and automation testing frameworks. Strong knowledge of programming languages such as Java, Python. Experience with test automation tools such as Selenium WebDriver. Familiarity with CI/CD tools like Jenkins, Git, or similar version control systems. Understanding of software development life cycle (SDLC) and testing methodologies. ( Note: Relevant applicants will receive an email requesting additional information as part of the next stage. The application process will be completed directly on the team's designated platform, and all subsequent communication and decisions regarding the opportunity are managed by the respective hiring team.)</t>
         </is>
@@ -778,21 +745,21 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Senior Software Development Engineer in Test</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/senior-software-development-engineer-in-test-at-experian-4445942915</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
         <is>
           <t>Experian</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E8" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -808,12 +775,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/senior-software-development-engineer-in-test-at-experian-4445942915</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Company Description Experian is a global data and technology company, powering opportunities for people and businesses around the world. We help to redefine lending practices, uncover and prevent fraud, simplify healthcare, create marketing solutions, and gain deeper insights into the automotive market, all using our unique combination of data, analytics and software. We also assist millions of people to realize their financial goals and help them save time and money. We operate across a range of markets, from financial services to healthcare, automotive, agribusiness, insurance, and many more industry segments. We invest in people and new advanced technologies to unlock the power of data. As a FTSE 100 Index company listed on the London Stock Exchange (EXPN), we have a team of 22,500 people across 32 countries. Our corporate headquarters are in Dublin, Ireland. Learn more at experianplc.com. Job Description Design, develop, and maintain automated test frameworks and scripts. Collaborate with development and QA teams to identify test requirements and create test plans. Execute automated tests and analyze results to identify defects and ensure software quality. Develop and maintain continuous integration and continuous deployment (CI/CD) pipelines. Work closely with development teams to ensure timely and effective testing of new features and bug fixes. Conduct code reviews and provide feedback to ensure code quality and adherence to best practices. Participate in sprint planning, daily stand-ups, and other Agile ceremonies. Investigate and troubleshoot issues in the test environments and escalate as necessary. You will report to an Engineering Manager Qualifications Bachelor's degree in computer science, Software Engineering, or a related field. You should hae 5+ years of experience as an SDET or in a similar role in software development and testing Experience with test automation tools and frameworks such as Playwright, Selenium, Appium, or similar. Strong programming skills in languages such as C#, Java, JavaScript, Python, Ruby Experience with agentic AI tools (GitHub Copilot, Cursor, Claude) and spec-driven agentic development. Test Planning (PBI Analysis, Establishing Priorities, Providing Estimates) Test Design (Create/Review Test Procedures, Create/Review Test Conditions, Identify/Create Test Data) Test Execution (Execute Test Procedures, Create/Triage Bugs, Status Reporting, Provide Requirements Traceability) Experience with XML and CSV formats for test data generation. Experience with UAT and Production implementation &amp; support. Validates Application Programming Interfaces (APIs), assuring the functionality, reliability, performance, and security of the programming interfaces Technical Aptitude in system interoperability procedures. Experience with SQL commands to create, store, retrieve, and modify data in a database Experience working with Agile/Scrum methodologies. Preferred Qualifications Advanced certifications such as ISTQB Certified Tester or similar. Experience with performance testing tools such as JMeter, LoadRunner, or similar. Familiarity with cloud platforms like Azure Additional Information Our uniqueness is that we celebrate yours. Experian's culture and people are important differentiators. We take our people agenda very seriously and focus on what matters; DEI, work/life balance, development, authenticity, collaboration, wellness, reward &amp; recognition, volunteering... the list goes on. Experian's people first approach is award-winning; World's Best Workplaces™ 2024 (Fortune Global Top 25), Great Place To Work™ in 24 countries, and Glassdoor Best Places to Work 2024 to name a few. Check out Experian Life on social or our Careers Site and Glassdoor to understand why. Experian is also proud to be an Equal Opportunity and Affirmative Action employer. If you have a disability or special need that requires accommodation, please let us know at the earliest opportunity. Recruitment Fraud Awareness - Experian's recruitment process is conducted only through authorised channels. Recruitment communications will only be sent from an @experian.com email address. Experian will never ask candidates to make any payment as part of an application, interview, assessment, onboarding, or recruitment process. To apply for roles or verify opportunities, please visit experian.com/careers. Benefits Experian care for employee's work life balance, health, safety and wellbeing. In support of this endeavor, we offer best-in-class family well-being benefits, enhanced medical benefits and paid time off. Experian Careers - Creating a better tomorrow together Find out what its like to work for Experian by clicking here</t>
         </is>
@@ -825,21 +787,21 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Enterprise Data Governance- Testing - Selenium, Java</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/enterprise-data-governance-testing-selenium-java-at-infosys-4472309222</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
         <is>
           <t>Infosys</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -855,12 +817,7 @@
           <t>Be among the first 25 applicants</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/enterprise-data-governance-testing-selenium-java-at-infosys-4472309222</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Selenium WebDriver Java TestNG / JUnit SQL Enterprise Data Governance Data Quality Testing API Testing (Postman/REST Assured) Git Agile Methodology Key Responsibilities Design, develop, and maintain automation frameworks using Selenium and Java. Create and execute automated test scripts for Data Governance applications. Validate data quality rules, metadata management, data lineage, and business glossary processes. Perform database testing using SQL queries. Test integrations between data governance, master data, and reporting systems. Validate data reconciliation, accuracy, completeness, and consistency. Execute API testing for governance-related services. Collaborate with Data Governance, Data Engineering, and Business teams. Participate in test planning, defect management, and release validation. Required Experience 3-5 years of experience in Automation Testing. Strong hands-on experience with Selenium WebDriver and Java. Experience in Data Governance, Data Quality, Metadata Management, or MDM projects. Strong SQL and database testing expertise. Knowledge of API testing tools. Experience with defect tracking tools such as JIRA. Understanding of Agile/Scrum methodologies. Experience with Informatica Data Governance, Collibra, Alation, Purview, or similar platforms. Knowledge of ETL/Data Warehouse testing. Exposure to cloud platforms (Azure, AWS, GCP). Familiarity with CI/CD tools such as Jenkins.</t>
         </is>
@@ -872,21 +829,21 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Quality Engineer I (Automation )</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/quality-engineer-i-automation-at-seismic-4398152163</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
         <is>
           <t>Seismic</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E10" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -902,12 +859,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/quality-engineer-i-automation-at-seismic-4398152163</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>About Us: Seismic is the Go-To-Market Performance company, driving how organizations turn their strategy into revenue. Seismic brings together signals from customer conversations, buyer engagement, governed content, coaching and seller behavior to turn intelligence into winning action. Through its AI revenue execution platform, the company equips customer-facing teams with the insights, governance, and contextual guidance they need to execute with confidence and deliver measurable business outcomes. Trusted by 2,500 organizations and over 3.5 million users around the globe, Seismic is headquartered in San Diego with offices across North America, Europe and Asia-Pacific. Learn more at seismic.com. Seismic is committed to building an inclusive workplace that ignites growth for our employees and creates a culture of belonging that allows all employees to be seen and valued for who they are. Learn more about DEI at Seismic here. Overview: Seismic is seeking a Software Engineer with 4+ years in Test with expertise in Python (or similar) to join our dynamic and innovative team.  As a key member of the Quality Engineering department, you will be responsible for ensuring the quality and reliability of our software products through the design, implementation, and execution of automated test suites and supporting test infrastructure and libraries. You will collaborate closely with developers, product managers, SRE, infrastructure, and delivery engineers to drive the development of scalable and robust software testing solutions. Who you are: Bachelor’s or Master’s degree in Computer Science or equivalent experience 4+ years of experience in software testing / quality engineering Strong experience in test automation Python preferred (Java or JavaScript automation experience also acceptable) Hands-on experience with Selenium or similar automation tools Strong understanding of testing principles, methodologies, and QA best practices Experience working with CI/CD pipelines (e.g., Jenkins, GitHub Actions) Experience with version control systems (GitHub) Exposure to tools like Jira, BrowserStack (or similar) Basic understanding or awareness of AI in testing (no deep ML expertise required) Good communication and collaboration skills Nice to have: Experience working in product-based companies Exposure to API or performance testing Familiarity with tools like New Relic, LaunchDarkly Understanding of Agile/Scrum methodologies What you’ll be doing: Design, develop, and maintain automated test scripts and frameworks (Python preferred) Perform functional testing across UI, API, and data layers Execute automated tests and analyze results to identify defects and areas for improvement Write test plans and test scenarios, and perform manual testing where required Collaborate with cross-functional teams to define test strategies and acceptance criteria Participate in design and coverage reviews to identify gaps and provide feedback Support defect triaging, debugging, and resolution Contribute to continuous improvement of testing processes and automation practices Leverage AI-assisted tools (e.g., Copilot or similar) to improve testing efficiency What we have for you: At Seismic, we’re committed to providing benefits and perks for the whole self. To explore our benefits available in each country, please visit the Global Benefits page. If you are an individual with a disability and would like to request a reasonable accommodation as part of the application or recruiting process, please click here. Seismic is an equal opportunity employer and all qualified applicants will receive consideration for employment without regard to gender, age, race, religion, or any other classification which is protected by applicable law. Please note this job description is not designed to cover or contain a comprehensive listing of activities, duties or responsibilities that are required of the employee for this job. Duties, responsibilities and activities may change at any time with or without notice. Please be aware we have noticed an increase in hiring scams potentially targeting Seismic candidates. Read our full statement on our Careers page.</t>
         </is>
@@ -919,21 +871,21 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Principal Engineer - Test Automation (CDMS)</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/principal-engineer-test-automation-cdms-at-veeva-systems-4437024311</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
         <is>
           <t>Veeva Systems</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>Mid-Senior level</t>
@@ -949,12 +901,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/principal-engineer-test-automation-cdms-at-veeva-systems-4437024311</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>Veeva Systems is a mission-driven organization and pioneer in industry cloud, helping life sciences companies bring therapies to patients faster. As one of the fastest-growing SaaS companies in history, we surpassed $3B in revenue in our last fiscal year with extensive growth potential ahead. At the heart of Veeva are our values: Do the Right Thing, Customer Success, Employee Success, and Speed. We're not just any public company – we made history in 2021 by becoming a public benefit corporation (PBC), legally bound to balancing the interests of customers, employees, society, and investors. Join us in transforming the life sciences industry, committed to making a positive impact on its customers, employees, and communities. The Role Do you dream about being part of a team with the talent, passion, and financial backing to build top-notch, industry-changing, cloud-based applications and platforms? At Veeva, we build enterprise cloud technology that powers the biggest names in pharmaceuticals, biotech, consumer goods, chemical &amp; cosmetics industries. Our customers make vaccines, life-saving medicines, and life-enhancing products that make a difference in everyday lives. Our technology has transformed these industries, enabling them to get critical products and services to market faster. Our products empower our customers in the fight against global pandemics like COVID-19. What You'll Do Learn and understand features of Veeva Vault platform and applications Work on CI/CD tools (Git, Jenkins, JIRA) on a daily basis Develop and maintain automation scripts (API and UI) Communicating status and working effectively with onshore/offshore managers Troubleshoot day to day technical issues related to test automation Perform code reviews and be a technical mentor to team members Work with managers to arrive at metrics for measuring the code quality for test automation suite Work closely with scrum masters on sprint plannings and backlog grooming Be a key player for the growth of Veeva Hyderabad by contributing to recruiting initiatives Requirements 10+ years of experience in software test automation Strong technical leadership abilities and project management experience Provide a practical approach to complex testing, specifically in the areas of the automation of test cases for the purposes of regression testing Proficient in QA process &amp; methodologies, tools, and different testing approaches Strong experience in Java, Object-Oriented Methodologies Strong experience with automated test frameworks (e.g., Selenium, Cucumber) Strong experience in testing Restful API &amp; HTTP web services, JSON/XML, and Web-based applications Good working knowledge of CI/CD tools (Git, Jenkins, JIRA) Experience in Mobile Testing and Automation – Appium, XCUI, Espresso, KI Experience in Mobile Apps Development (Android/iOS) Experience with data analytics and log analysis tools such as Kibana, Elasticsearch, etc. Able to lead multiple implementations Collaborate to gather automation requirements, design automated tests and implement scalable test automation solutions Design, develop and manage automated testing artifacts Comfortable debugging and working with object-oriented programming Experience with Agile/Scrum development methodologies (preferably in an onshore /offshore model) Experience working for a product-based company Excellent team collaboration and effective communication skills Experience playing a technical mentor role to the team and performing code reviews Experience leading automation projects in a technical role and actively participating in overall program/project management activities Experience with applicable software and programs, including Kotlin, Swift, JAVA, and React Fluency in interfacing and functional testing A natural problem solver and critical thinker Knowledge of modern best practices for software development, including IDE, source control, build processes, release management, and deployment Bachelor’s or Master’s Degree in Computer Engineering, Computer Science, Electrical Engineering, or similar Nice to Have Experience with Android and Mac platforms Perks &amp; Benefits Health insurance with generous coverage limits Fixed bonus Allowance for wellness &amp; fitness programs Winter break Veeva’s headquarters is located in the San Francisco Bay Area with offices in more than 15 countries around the world. Veeva is an equal opportunity employer. All qualified applicants will receive consideration for employment without regard to race, color, sex, sexual orientation, gender identity or expression, religion, national origin or ancestry, age, disability, marital status, pregnancy, protected veteran status, protected genetic information, political affiliation, or any other characteristics protected by local laws, regulations, or ordinances.</t>
         </is>
@@ -966,21 +913,21 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>PQE II</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/pqe-ii-at-phenom-4473773892</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
         <is>
           <t>Phenom</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -996,12 +943,7 @@
           <t>80 applicants</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/pqe-ii-at-phenom-4473773892</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Job Requirements Role Overview We are looking for a highly skilled Senior SDET (PQE II) with strong expertise in Automation Testing using Playwright with Java/Python . The ideal candidate will be responsible for building scalable automation frameworks, driving quality engineering best practices, and mentoring junior QA engineers. This role requires deep understanding of test automation architecture, CI/CD integration, API testing, and performance validation within Agile environments. Key Responsibilities Design, develop, and maintain robust automation frameworks using Playwright (Java or Python) Build scalable, reusable, and maintainable test automation suites for Web and API applications Integrate automation pipelines with CI/CD tools (Jenkins/GitHub Actions/Azure DevOps) Develop automation for REST APIs using tools like RestAssured / PyTest Work closely with developers and product teams to define acceptance criteria and test strategies Perform root cause analysis and identify automation gaps Improve test execution performance and optimize framework stability Participate in sprint planning, grooming, and release validation Technical Skills Required Mandatory Skills 4+ years of experience in QA Automation / SDET role Strong hands-on experience in Selenium WebDriver Strong hands-on experience in Playwright Proficiency in Java or Python (OOPS concepts mandatory) Experience in building automation frameworks from scratch (Hybrid / POM / BDD) Experience in API automation testing CI/CD integration experience Strong SQL knowledge Experience working in Agile/Scrum environments Good to Have Experience with Docker/Kubernetes Performance testing exposure (JMeter / Gatling) Cloud platform exposure (AWS/Azure/GCP) Security testing basics Experience with Test Management tools (Jira, Zephyr, TestRail) Behavioral Competencies Strong analytical and problem-solving skills Excellent communication and stakeholder management Ownership mindset with high accountability Ability to drive quality improvements independently What We Expect From PQE III Level Ability to independently design automation strategy Mentor team members and review automation code Identify quality risks early and provide mitigation plans Contribute to engineering best practices and reusable components</t>
         </is>
@@ -1013,21 +955,21 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Engineer II, Software Dev Test QE</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/engineer-ii-software-dev-test-qe-at-lpl-financial-global-capability-center-4465022012</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
         <is>
           <t>LPL Financial Global Capability Center</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Greater Hyderabad Area</t>
-        </is>
-      </c>
       <c r="E13" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -1043,12 +985,7 @@
           <t>111 applicants</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/engineer-ii-software-dev-test-qe-at-lpl-financial-global-capability-center-4465022012</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>Where Ambition Meets Innovation At LPL’s Global Capability Center, you'll find a collaborative culture where your voice matters, integrity guides every decision, and technology fuels progress. Your skills, talents, and ideas will redefine what's possible. LPL's success reflects its exceptional employees, who together pursue one noble purpose: empowering financial advisors to deliver personalized advice for all who need it. We’re proud to be expanding and reaching new heights in Hyderabad. Join us as we create something extraordinary together. Are you passionate about driving positive outcomes through effective technology? Do you thrive on complex initiatives and bringing new ideas to life? Excited to learn more? If so, then this could be the role for you! LPL Financial (Nasdaq: LPLA) was founded on the principle that the firm should work for the advisor, and not the other way around. Today, LPL is a leader* in the markets we serve, supporting more than 18,000 financial advisors, 800 institution-based investment programs and 450 independent RIA firms nationwide. We are steadfast in our commitment to the advisor-centered model and the belief that Americans deserve access to personalized guidance from a financial advisor. At LPL, independence means that advisors have the freedom they deserve to choose the business model, services, and technology resources that allow them to run their perfect practice. And they have the freedom to manage their client relationships because they know their clients best. Simply put, we take care of our advisors, so they can take care of their clients. What are we looking for? We are seeking highly skilled individuals to join our Corporate Systems engineering team, capable of delivering outstanding client experiences. This role requires close collaboration with our platform technical lead, Architects, DBA and Release Management to deliver testing solutions that align with business requirements. The Corporate Systems engineering team is committed to providing high-quality solutions and data to its users on a large scale. Ideal candidates should possess relevant practical experience and demonstrate proficiency in working within an enthusiastic team environment. Ideal candidate should be dynamic, continuous learners who exhibit curiosity and strive for success in a fast-paced setting, emphasizing results, teamwork, innovation, and continuous improvement. Engineer II, Software Dev Test QE As a Quality Engineer, you will be responsible for comprehensive testing, coordinating releases, and providing outstanding support to meet business needs. Collaborating with the Corporate Systems Tech Lead, Architects, QA, and Release Management teams, you'll contribute to developing an application that supports our business objectives. Our department focuses on delivering robust, large-scale data integration and innovative home office solutions. We seek candidates with practical experience, a commitment to ongoing learning, and a passion for teamwork and excellence. Primary Duties And Responsibilities Design, develop and execute manual and automated test cases for custom web-based application, APIs and ETLs. Ensure end-to-end quality by implementing testing strategies, automation frameworks, and best practices. Work closely with developers, product owners and business stakeholders to align testing efforts with project requirements. Collaborate in Agile environments, actively participating in requirements gathering, sprint planning, and daily stand-ups. Continuously improve testing processes, identify gaps and implement automation where feasible. Communicate on team's behalf to both technical and non-technical audiences. Work in an agile environment with various scrum teams, using test management tools such as Zephyr. Support planned change requests and releases. Knowledge &amp; Experience 4+ years of experience in information technology/software development with a proven ability to ensure high quality results and with expertise in test automation, agile methodologies and QA best practices. 4+ years of hands-on experience in Selenium, TestNG, Cucumber and PowerShell for automation. 2+ years in SQL development. Solid knowledge of QA methodologies, test planning, system dependencies, and product integration phases Experience with Atlassian tool set, JIRA, Confluence, etc. Experience with AI in software testing/development. Experience with root cause analysis and problem solving. Core Competencies C#, .Net, Java, SQL, Cursor AI, GitHub CoPilot, Test Automation Tool, PowerShell, and Linux Strong analytical and problem-solving skills. Tumbleweed, Octopus, Sonar, Git, Swagger, Postman, and AWS. Experience with Waterfall and Agile development process. Excellent verbal and written communication skills. Preferences Bachelor’s degree in computer science, or a related field Experience with Snowflake, Oracle Autonomous Data Warehouse, Tableau or Power BI is a plus. Familiar with FinOps. Experience with Data analytic processes and tools is a plus. Excellent knowledge of OOP concepts, data modeling and design patterns/frameworks. LPL Global Business Services, LLP - PRIVACY POLICY</t>
         </is>
@@ -1060,21 +997,21 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Automation Test Lead</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/automation-test-lead-at-birlasoft-4472120906</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
         <is>
           <t>Birlasoft</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E14" t="inlineStr">
         <is>
           <t>Mid-Senior level</t>
@@ -1090,12 +1027,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/automation-test-lead-at-birlasoft-4472120906</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>Experience- 7- 10 years Location- Hyderabad- Notice period- Immediate JD- Strong experience in software quality engineering, test strategy, test planning, and QA leadership across enterprise applications. Expertise in UI automation testing using Selenium and Playwright or equivalent frameworks. Experience designing and implementing test automation frameworks using Java, Python, JavaScript, or similar technologies. Strong experience in functional, integration, regression, system, and end-to-end testing. Strong knowledge of Agile/Scrum, Shift-Left Testing, Continuous Testing, and Quality Engineering practices. Strong understanding of JSON, XML, REST APIs, SOAP, web services, and microservices architectures. Strong experience with cloud environments, preferably Pivotal Cloud Foundry and/or AWS/Azure/GCP. Knowledge of Splunk or equivalent production monitoring tools for log analysis, troubleshooting, and root-cause identification. Experience establishing QA metrics, quality gates, defect management, test coverage, and release-readiness criteria. Ability to lead test automation strategy and framework modernization, reducing manual testing and improving release velocity. Strong experience in AI-led Quality Engineering, leveraging AI/GenAI capabilities to improve test planning, test design, automation, execution, defect analysis, and overall software quality. Preferably generating test case and script creation using copilot. Experience using AI-assisted test generation and automation tools to generate test scenarios, test cases, automation scripts, regression suites, and test data. Experience leveraging AI/GenAI for defect analysis, root-cause analysis, log analysis, failure prediction, and intelligent test prioritization. Experience evaluating and adopting AI-powered QA/testing tools to improve testing efficiency, coverage, productivity, and quality. Hands-on experience with AI development/productivity tools such as GitHub Copilot or equivalent AI tools, with the ability to apply them effectively in QA automation and Quality Engineering activities. Ability to identify opportunities where AI can replace or augment repetitive manual QA activities and drive measurable improvements in automation and productivity. Understanding of AI/ML application testing, including validation of AI-driven functionality, data quality, model behavior, accuracy, reliability, and edge cases, where applicable. Experience mentoring QA engineers and providing technical leadership across distributed and cross-functional teams. Strong collaboration skills with Development, Product, Architecture, DevOps, and Business teams. Excellent technical communication skills with the ability to communicate effectively with technical and non-technical stakeholders. Strong analytical and problem-solving skills with the ability to identify root causes, assess impact, define action plans, and drive issues to closure. Experience delivering quality solutions in financial/banking applications is preferred. Strong attention to detail and ability to work effectively in a dynamic, fast-paced environment.</t>
         </is>
@@ -1107,21 +1039,21 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>Senior Quality Assurance Automation Engineer</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/senior-quality-assurance-automation-engineer-at-zapcom-group-inc-4460602935</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
         <is>
           <t>Zapcom Group Inc</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E15" t="inlineStr">
         <is>
           <t>Mid-Senior level</t>
@@ -1137,12 +1069,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/senior-quality-assurance-automation-engineer-at-zapcom-group-inc-4460602935</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>Role: QA Automation Engineer Location: Hyderabad/Bangalore, India Work Type: Onsite Minimum experience required is 8+ Years The client is looking for strong QA Automation candidates with hands-on experience in test automation and modern testing frameworks. Key expectations: Strong experience in QA Automation testing Experience designing and maintaining automation frameworks Hands-on experience with Selenium, Cypress, Playwright, or similar automation tools Programming knowledge in Java, Python, or JavaScript Experience with API testing (Postman, Rest Assured, etc.) Strong understanding of Software Testing Life Cycle (STLC) and Agile methodologies Experience writing and executing automated test cases Knowledge of regression, functional, integration, and end-to-end testing Experience with CI/CD tools such as Jenkins, GitHub Actions, or similar Strong debugging and defect tracking skills Experience using tools like JIRA, TestRail, or similar Database testing and SQL knowledge preferred Good communication skills and ability to work closely with developers and business teams Please focus on strong hands-on automation experience and can clearly explain the frameworks, tools, and automation solutions they have implemented in their projects. About Us Zapcom Zapcom is a global technology services company focused on crafting meaningful digital solutions that transform businesses. Driven by agility, innovation, and a customer-first mindset, we work with clients across the US, India, Europe, Canada, and the MENA region . We specialize in building modern platforms and digital products for industries such as airlines, travel, hospitality, BFSI, retail, and healthcare . Our product-first approach means we think like product owners, design like architects, and test like customers—ensuring scalable, high-quality solutions. Our builder-led culture and dual-factory delivery model enable us to deliver impact at speed, grounded in ownership, transparency, and focused execution. At Zapcom, you’re trusted to lead, encouraged to take initiative, and empowered to shape solutions that are used by millions worldwide. If you’re someone who thrives on responsibility, enjoys solving real-world problems, and steps up when it matters, you’ll feel right at home here. Join us and help shape products and experiences that make a global impact.</t>
         </is>
@@ -1154,21 +1081,21 @@
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Senior Software Developer Engineer in Test</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/senior-software-developer-engineer-in-test-at-experian-4473952413</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
         <is>
           <t>Experian</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E16" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -1184,12 +1111,7 @@
           <t>57 applicants</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/senior-software-developer-engineer-in-test-at-experian-4473952413</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>Company Description Experian is a global data and technology company, powering opportunities for people and businesses around the world. We help to redefine lending practices, uncover and prevent fraud, simplify healthcare, create marketing solutions, and gain deeper insights into the automotive market, all using our unique combination of data, analytics and software. We also assist millions of people to realize their financial goals and help them save time and money. We invest in people and new advanced technologies to unlock the power of data. As a FTSE 100 Index company listed on the London Stock Exchange (EXPN), we have a team of 25,200 people across 32 countries. Our corporate headquarters are in Dublin, Ireland. Learn more at experianplc.com. Job Description We are looking for an enthusiastic Test Engineer to work at the forefront of our cloud modernisation, within our Credit &amp; Verification Services. This is a hybrid role requiring travelling to Hyderabad office circa 40% days per month. Role Context We're predominantly a .NET focused engineering team, building modern, cloud-native applications using the latest in .NET 8+. All new services are developed with a forward-looking mindset, and we actively evaluate emerging features and tools to continuously improve our engineering practices. Our architecture is built on Kubernetes (EKS), enabling us to run scalable, resilient microservices in the cloud. On top of this, we leverage a wide range of AWS services (Lambda, Kinesis, Dynamo and RDS to name just a few), to enhance performance, observability, and integration across our platform. Key Responsibilities Design, develop, and execute manual and automated test scripts based on business requirements. Develop, maintain, and enhance automation frameworks for UI, API, and backend testing. Create and maintain test data, test environments, and automation scripts. Perform various types of testing: White Box testing, Black Box testing, Integration testing,UI testing, API Testing Qualifications 4+ years of experience in a quality engineering, software testing, or test automation. Experience with SDLC, STLC, and Agile/Scrum processes. You will work collaboratively in cross-functional teams. Passion for quality, learning new technologies, and continuous improvement. Hands-on experience with UI, API automation tools like Selenium, Cypress, Playwright, REST-assured or Postman. Proficiency in Behaviour-Driven Development (BDD) and Test-Driven Development (TDD) approaches. Working knowledge of SQL for data validation. Experience in at least one programming/scripting language: Java, Scala, Python, or JavaScript. Basic understanding of Containers (Docker) and CI/CD processes. Experience with version control systems like Git, Bitbucket, GitHub or Gitlab. Working knowledge of API testing, backend validations, and functional automation. You will report to manager. Additional Information Our uniqueness is that we celebrate yours. Experian's people first approach is award-winning; World's Best Workplaces™ 2025 (Fortune Top 25), Great Place To Work™ in 26 countries to name a few. Check out Experian Life on social or our Careers Site to understand why. Experian is proud to be an Equal Opportunity and Affirmative Action employer. Innovation is an important part of Experian's DNA and practices, and our diverse workforce drives our success. Everyone can succeed at Experian and bring their whole self to work, irrespective of their gender, ethnicity, religion, colour, sexuality, physical ability or age. If you have a disability or special need that requires accommodation, please let us know at the earliest opportunity. Recruitment Fraud Awareness - Experian's recruitment process is conducted only through authorised channels. Recruitment communications will only be sent from an @experian.com email address. Experian will never ask candidates to make any payment as part of an application, interview, assessment, onboarding, or recruitment process. To apply for roles or verify opportunities, please visit experian.com/careers. Benefits Experian care for employee's work life balance, health, safety and wellbeing. In support of this endeavor, we offer best-in-class family well-being benefits, enhanced medical benefits and paid time off. Experian Careers - Creating a better tomorrow together Find out what its like to work for Experian by clicking here Experian Careers - Creating a better tomorrow together Find out what its like to work for Experian by clicking here</t>
         </is>
@@ -1201,21 +1123,21 @@
           <t>2026-09-29</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>Senior Quality Assurance Automation Engineer</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/senior-quality-assurance-automation-engineer-at-gaian-solutions-4470852287</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
         <is>
           <t>Gaian Solutions</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E17" t="inlineStr">
         <is>
           <t>Mid-Senior level</t>
@@ -1231,12 +1153,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/senior-quality-assurance-automation-engineer-at-gaian-solutions-4470852287</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>About the Role We are looking for an experienced Automation QA Engineer to join our team. The ideal candidate combines strong QA fundamentals with solid programming skills, and has some hands-on development exposure. You will design, build, and maintain automation frameworks, and help ensure the quality of cloud-hosted applications. Key Responsibilities Design, develop, and maintain automated test suites using Robot Framework. Create custom Python keywords and libraries to extend Robot Framework. Analyze requirements and create test plans, test cases, and test data for functional, regression, integration, and end-to-end testing. Test applications deployed on AWS and validate behavior across environments. Integrate automated tests into CI/CD pipelines (Jenkins, GitLab CI, GitHub Actions, or AWS Code Pipeline). Perform API testing and backend validation. Identify, log, and track defects, and work with developers to resolve them. Review automation code, mentor junior team members, and promote QA best practices. Contribute to improving test coverage, execution speed, and framework reliability. Required Skills 7-8 years of experience in software testing, with a strong focus on test automation. Strong hands-on experience with Robot Framework and Selenium for web UI automation. Proficiency in Python (or Java) for scripting and framework development. Some experience in software development, with the ability to read and debug application code. Experience with API testing (Postman, REST Assured, or Robot Framework Requests Library). Working knowledge of AWS services (EC2, S3, Lambda, RDS, CloudWatch, API Gateway). Experience with CI/CD tools and version control (Git). Good SQL skills for database validation. Solid understanding of the SDLC, STLC, and Agile/Scrum methodologies. Strong analytical, debugging, and communication skills. Experience with Docker and containerized test execution. Exposure to performance testing (JMeter, Locust). Experience with Infrastructure as Code (Terraform, CloudFormation). Familiarity with BDD (Behave, Cucumber) and test management tools (Jira, TestRail, Zephyr). Good to Have AWS certification (Cloud Practitioner or higher). Qualifications Bachelor's degree in Computer Science, Engineering, or a related field. Additional Requirements Ability to join immediately. Ability to work independently and in a collaborative team environment. Notice Period: Immediate joiner preferred</t>
         </is>
@@ -1248,21 +1165,21 @@
           <t>2026-09-29</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>QA Automation Engineer</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/qa-automation-engineer-at-lseg-4471707958</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
         <is>
           <t>LSEG</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E18" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -1278,12 +1195,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/qa-automation-engineer-at-lseg-4471707958</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>Future Talent: QA Automation Engineer (Talent Community – India) Location: Bengaluru / Hyderabad Position Type: Future Opening – Talent Pipeline The Opportunity We are continuously searching for exceptional QA Automation Engineers across India to help us deliver high-quality, scalable, and reliable software solutions. While we may not have an immediate opening today, this dedicated QA Talent Community helps us engage with top testing professionals early. By joining our engineering community, you'll gain insights into our quality engineering practices, automation strategy, engineering culture, and events, and be among the first to be considered when matching opportunities arise. What You'll Do (When You Join Us) As a QA Automation Engineer , you will work on enterprise-grade applications, ensuring software quality through automation, continuous testing, and engineering excellence. Design &amp; Automate Design, develop, and maintain automated test frameworks and test solutions. Build scalable automation for functional, regression, integration, and API testing. Improve test coverage and efficiency through automation best practices. Quality &amp; Excellence Validate application functionality, performance, reliability, and user experience. Identify defects early and collaborate with engineering teams to resolve issues. Support CI/CD and continuous testing initiatives. Collaborate Work in an Agile environment with developers, product owners, architects, and platform teams. Participate in solution reviews, sprint activities, and quality discussions. Contribute to engineering best practices and continuous improvement initiatives. What You'll Bring Strong experience in Software Testing and QA Automation. Experience with automation tools and frameworks such as Selenium, Playwright, Cypress, PyTest, or similar. Proficiency in one or more programming languages such as Java, Python, C#, or JavaScript. Experience with API, database, and end-to-end testing. Familiarity with Agile methodologies and CI/CD practices. Strong analytical, problem-solving, and communication skills. Passion for quality engineering, automation, and continuous learning. What You'll Bring Beyond Skills Build With Purpose – Focus on delivering quality outcomes. Customer Driven – Advocate for exceptional user experiences. Learn and Be Curious – Continuously develop your expertise. Act as Owner – Take responsibility for software quality. Lead with Data – Use evidence and metrics to drive decisions. Collaborate to Achieve – Work openly and effectively across teams. How We Hire Our process is skills-focused and designed to be fair and consistent. Candidates may complete technical assessments and interviews focused on automation, quality engineering, problem-solving, and collaboration. Why Connect Now? Skip the Line Candidates in this talent community are prioritised for evaluation when suitable QA opportunities become available. Exclusive Insights Receive invitations to engineering events, webinars, and technology discussions. Career Alignment We connect with candidates for roles that match their interests in automation testing, quality engineering, platform testing, API testing, performance testing, and continuous quality practices. How To Join Upload your CV along with a short note about: Your QA and automation experience. Preferred testing technologies and tools. Areas of interest such as Automation Testing, API Testing, Performance Testing, Quality Engineering, or Test Framework Development. We will review your profile and connect for an informal conversation to better understand your interests and career aspirations. Proud to share LSEG in the India is Great Place to Work certified (Jun ’25 – Jun ’26). Career Stage: Senior Associate London Stock Exchange Group (LSEG) Information: Join us and be part of a team that values innovation, quality, and continuous improvement. If you're ready to take your career to the next level and make a significant impact, we'd love to hear from you. LSEG is a leading global financial markets infrastructure and data provider. Our purpose is driving financial stability, empowering economies and enabling customers to create sustainable growth. Our purpose is the foundation on which our culture is built. Our values of Integrity, Partnership , Excellence and Change underpin our purpose and set the standard for everything we do, every day. They go to the heart of who we are and guide our decision making and everyday actions. Working with us means that you will be part of a dynamic organisation of 25,000 people across 65 countries. However, we will value your individuality and enable you to bring your true self to work so you can help enrich our diverse workforce. We are proud to be an equal opportunities employer. This means that we do not discriminate on the basis of anyone’s race, religion, colour, national origin, gender, sexual orientation, gender identity, gender expression, age, marital status, veteran status, pregnancy or disability, or any other basis protected under applicable law. Conforming with applicable law, we can reasonably accommodate applicants' and employees' religious practices and beliefs, as well as mental health or physical disability needs. You will be part of a collaborative and creative culture where we encourage new ideas. We are committed to sustainability across our global business and we are proud to partner with our customers to help them meet their sustainability objectives. Our charity, the LSEG Foundation provides charitable grants to community groups that help people access economic opportunities and build a secure future with financial independence. Colleagues can get involved through fundraising and volunteering. LSEG offers a range of tailored benefits and support, including healthcare, retirement planning, paid volunteering days and wellbeing initiatives. Please take a moment to read this privacy notice carefully, as it describes what personal information London Stock Exchange Group (LSEG) (we) may hold about you, what it’s used for, and how it’s obtained, your rights and how to contact us as a data subject. If you are submitting as a Recruitment Agency Partner, it is essential and your responsibility to ensure that candidates applying to LSEG are aware of this privacy notice.</t>
         </is>
@@ -1295,21 +1207,21 @@
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>Senior Technical Consultant- QA Automation</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/senior-technical-consultant-qa-automation-at-perficient-4472754780</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
         <is>
           <t>Perficient</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E19" t="inlineStr">
         <is>
           <t>Mid-Senior level</t>
@@ -1325,12 +1237,7 @@
           <t>59 applicants</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/senior-technical-consultant-qa-automation-at-perficient-4472754780</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>This position is for our Nagpur, Pune, Chennai, Hyderabad, Bangalore offices and you are expected to work out any of these locations only. Design, develop, and execute manual test plans and scripts to test the functionality of AEM websites. Must have worked on Java -Selenium automation experience. AEM with Automation QA experience will be highly preferred In depth, functional, regression testing of new or enhanced features in the AEM 6.5 environment. Expertise in AEM- Forms, Sites, Assets and DAM. Expertise in AEM -Experience fragments and Content Fragment. Good hands-on knowledge on MSM related concepts Good to have Java -Selenium automation experience. Should be excellent in writing functional and technical documentation. Must have strong analytical skills and should be detail oriented. Good communication, interpersonal, presentation, and problem-solving skills. Select work authorization questions to ask when applicants apply 1. Are you legally authorized to work in the United States? 2. Will you now, or in the future, require sponsorship for employment visa status (e.g. H-1B visa status)?</t>
         </is>
@@ -1342,21 +1249,21 @@
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>SDET Senior Test Lead</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/sdet-senior-test-lead-at-hcltech-4470847982</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
         <is>
           <t>HCLTech</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E20" t="inlineStr">
         <is>
           <t>Mid-Senior level</t>
@@ -1372,12 +1279,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/sdet-senior-test-lead-at-hcltech-4470847982</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>Job description: Skill Requirements 1. Experience in api testing and webservices testing 2. Proficiency in automated testing tools such as selenium 3. Good understanding of sdet (software development engineer in test) principles 4. Solid programming skills in languages such as java, python, or javascript 5. Knowledge of software development lifecycle and agile methodologies 6. Ability to work collaboratively in a team environment 7. Strong analytical and problem-solving abilities 8. Good communication skills to interact with cross functional teams Must Have Skills Click Enter to show the proficiency description of Software Development Engineer in Test (SDET)Software Development Engineer in Test (SDET) Click Enter to show the proficiency description of API TestingAPI Testing Click Enter to show the proficiency description of SeleniumSelenium Click Enter to show the proficiency description of PlaywrightPlaywright Click Enter to show the proficiency description of JavaScriptJavaScript Profile description: Skill Requirements 1. Experience in api testing and webservices testing 2. Proficiency in automated testing tools such as selenium 3. Good understanding of sdet (software development engineer in test) principles 4. Solid programming skills in languages such as java, python, or javascript 5. Knowledge of software development lifecycle and agile methodologies 6. Ability to work collaboratively in a team environment 7. Strong analytical and problem-solving abilities 8. Good communication skills to interact with cross functional teams Must Have Skills Click Enter to show the proficiency description of Software Development Engineer in Test (SDET)Software Development Engineer in Test (SDET) Click Enter to show the proficiency description of API TestingAPI Testing Click Enter to show the proficiency description of SeleniumSelenium Click Enter to show the proficiency description of PlaywrightPlaywright Click Enter to show the proficiency description of JavaScriptJavaScript</t>
         </is>
@@ -1389,21 +1291,21 @@
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Senior Quality Engineer</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/senior-quality-engineer-at-huntingcube-4472782124</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
         <is>
           <t>HuntingCube</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E21" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -1419,12 +1321,7 @@
           <t>167 applicants</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/senior-quality-engineer-at-huntingcube-4472782124</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>Job Description Responsibilities: - Develop, publish, manage, and execute test strategies, test plans, test cases, traceability matrices, automation scripts, status reports, defect logs, and exit reports. - Identify and obtain required test data and test environments. - Develop, publish, and manage testing estimates and financials. - Manage and lead the testing activities of a workstream, program, or multiple projects/initiatives. - Build team and individual capabilities by providing development opportunities such as special projects and training. - Ensure adherence to QA/QE standards and support the implementation of new standards. - Recognize and identify areas where policies, processes, procedures, tools/methodologies need to be changed or developed or can be improved. Identify and implement continuous improvements. - Track and report QA/QE metrics and KPIs such as velocity, defect slippage, etc. - Identify, manage, and implement remediation for any noncompliance items and deviations. - Provide technical input and feedback on design, assess impact on testing, and find QA automation solutions based on the solution being implemented. - Identify and implement automation, AI, or other emerging solutions to expedite testing, improve quality, and reduce costs. - Apply extensive knowledge of software quality assurance, quality management, and problem-solving methodologies. Requirements: - 3-5 years of experience in QA/QE, 1-3 years of experience in development. - Bachelor's degree in computer science, Engineering, Information Technology, or a related field. - Retail banking, mobile testing, web-based testing, UX testing, API testing, Accessibility. Must Have Skills: - Coordination skills - create and execute test plans, test cases, and traceability matrices. - Web services and/or APIs. - Database testing - basic SQL knowledge. - Experience in evaluating systems, software packages, and tools for functionality and quality requirements. - Strong understanding of quality management methods, tools, and techniques. - Strong verbal and written communication skills. - Problem-solving skills and ability to resolve operational or process issues. - Writing and executing automation test cases, custom functions, and building object repositories for web and native page elements. Good to have Skills: - Automation scripting Language: Python (Python + Java). - Good to have skills: ETL testing. UNIX testing skills, GRPC. - Proficiency with Jira, Confluence, and/or other similar Agile, development, and QA tools. - Automation frameworks, tools, and libraries: Selenium WebDriver, Appium, TestNG, Junit. - Version control systems for code management, e. g., Git. - Web technologies: HTML, CSS, web services. - GitHub Copilot or other Gen AI-based tools. - Perfecto and/or other mobile and browser testing tools. - Parasoft, Postman, Swagger / OpenAI, Insomnia, or any other similar tools. Company Summary GCCX is the platform to build and scale global teams in India faster, smarter, and without the chaos. We bring insights, talent, and operations together so startups and SMBs can launch in under 90 days and grow with confidence. Pods that launch GTMs in weeks. Capabilities that unlock scale. Agentic and human teams that just deliver. Global founders are already building in India to access top talent without burning a hole in their pocket. Helping global businesses make India their advantage! Make it possible for companies to do more with fewer, better teams, faster execution, and longer runways. We've built in India. Scaled in India. Now, we're helping businesses do the same faster, cleaner, and smarter. Why Join Us Outcomes and opportunities are what we value. We trust our team members and believe they work with us because they believe in the mission of creating a million global jobs in India by 2030 That can be done from anywhere! Required Skills ['API', 'Appium', 'Python', 'QA', 'QE', 'SQL', 'Selenium', 'automation', 'quality assurance', 'quality engineering', 'test automation', 'testing'] Additional Information Source recruiter: Karthik N V Source recruiter designation: Senior Talent Scout Company tagline: Build teams and GCCs across India Employee count: 10 Company founded: 2024 Benefits: Remote working options, Non-linear workdays Website: https://gccxglobal.com/ LinkedIn: https://www.linkedin.com/company/gccx/about/ Instahyre score: 1 Strong match: true Accept outstation: true Company tagline: Build teams and GCCs across India Logo: https://media.instahyre.com/images/profile/base/employer/53312/6742b53ca1/gccx_logo.webp</t>
         </is>
@@ -1436,21 +1333,21 @@
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>Senior Software Engineering Lead - React UI Automation</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/senior-software-engineering-lead-react-ui-automation-at-optum-india-4473021622</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
         <is>
           <t>Optum India</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E22" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -1466,12 +1363,7 @@
           <t>137 applicants</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/senior-software-engineering-lead-react-ui-automation-at-optum-india-4473021622</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>Optum is a global organization that delivers care, aided by technology to help millions of people live healthier lives. The work you do with our team will directly improve health outcomes by connecting people with the care, pharmacy benefits, data and resources they need to feel their best. Here, you will find a culture guided by inclusion, talented peers, comprehensive benefits and career development opportunities. Come make an impact on the communities we serve as you help us advance health optimization on a global scale. Join us to start Caring. Connecting. Growing together. Primary Responsibilities Develop and deliver applications using modern UI frameworks and scalable backend microservices under established architectural guidelines Design, implement, test, and troubleshoot software components and features, ensuring quality, performance, and reliability Develop micro‑products and services using React / Nextjs for front‑end and Spring Boot / Python for backend development Contribute to building AI‑enabled features, including exposure to Generative AI and agent‑based workflows, under guidance from senior engineers Develop and enhance user interfaces using modern JavaScript frameworks, with a focus on usability, performance, and maintainability Write and optimize database queries and stored procedures using MS SQL and work with GraphQL APIs for efficient data access Collaborate as part of an Agile/Scrum team to deliver new product features and services in iterative release cycles Participate actively in code reviews, following coding standards and incorporating feedback to improve code quality Support and improve CI/CD pipelines, contributing to build, deployment, and automation efforts for cloud‑native applications Build automated tests for UI/ backend/ APIs Write and execute automated tests in a TDD (Test Driven Development) setup Manage test data for Automation Engineer solutions that collect and report test results through various metrics reporting tools, example Sonar Demonstrate expertise in black box and grey box testing methodologies, experience with standard QA and development tools, and the ability to operate within short release cycles Develop in-depth system and product knowledge Constantly evaluate the test automation strategy and approach to identify areas of improvement (i.e. test automation frameworks, dynamic data collection methodologies, coding standards, components and object repository methods, etc.) Assist and mentor Automation QA testers in learning and developing automated scripts. Provide recommendations for improvement and share explanations and information to support team development Document and mentor Quality engineers on the use of the testing framework Partner with product owners and developers to identify areas for improved efficiencies Research and implement tools to support delivery Assist with DevOps support Comply with the terms and conditions of the employment contract, company policies and procedures, and any and all directives (such as, but not limited to, transfer and/or re-assignment to different work locations, change in teams and/or work shifts, policies in regards to flexibility of work benefits and/or work environment, alternative work arrangements, and other decisions that may arise due to the changing business environment). The Company may adopt, vary or rescind these policies and directives in its absolute discretion and without any limitation (implied or otherwise) on its ability to do so Required Qualifications Undergraduate degree or equivalent experience 10+ years of hands‑on experience in application development, with practical exposure to React‑based UI, Java/Spring Boot microservices, and API‑driven architectures Experience contributing to reusable backend services or shared components (such as workflows, rules, orchestration, or data services) that are used by more than one application or team Hands on Experience with Test automation frameworks - Selenium, Playwright, Cypress or similar Experience to define and report Quality Engineering metrics Experience to lead and mentor a team of Quality engineers Good understanding of building secure, reliable, and scalable systems, including basics of authentication/authorization, performance considerations, logging/monitoring, and supporting applications in production environments Practical exposure to applying AI/ML or NLP concepts to real‑world problems such as automation, API onboarding an consumption, or decision support, under guidance from senior engineers API testing/ Automation - Postman/ Rest Assured/ Karate or similar experience Cross browser testing / automation using Sauce Labs/ Browser Stack or similar experience Solid expertise building Scenarios with BDD frameworks - Cucumber, Spec flow or similar Demonstrated delivery of solutions that promote code reuse, maintainability, and faster development, beyond one‑off or tightly coupled implementations Proven solid Coding skills - Java/ Jscript, Typescript or similar Willingness and ability to learn, collaborate, and receive mentorship, while sharing knowledge with peers and following engineering best practices across platform and AI‑enabled components Demonstrated ability to design and build test automation frameworks from scratch - choosing right frameworks based on project needs Demonstrated ability to work in a flexible/ fast paced Agile environment Proven solid communication skills, problem solving skills At UnitedHealth Group, our mission is to help people live healthier lives and make the health system work better for everyone. We believe everyone-of every race, gender, sexuality, age, location and income-deserves the opportunity to live their healthiest life. Today, however, there are still far too many barriers to good health which are disproportionately experienced by people of color, historically marginalized groups and those with lower incomes. We are committed to mitigating our impact on the environment and enabling and delivering equitable care that addresses health disparities and improves health outcomes - an enterprise priority reflected in our mission.</t>
         </is>
@@ -1483,21 +1375,21 @@
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>Software Development Engineer in Test</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/software-development-engineer-in-test-at-the-depository-trust-clearing-corporation-dtcc-4464375176</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
         <is>
           <t>The Depository Trust &amp; Clearing Corporation (DTCC)</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E23" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -1513,12 +1405,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/software-development-engineer-in-test-at-the-depository-trust-clearing-corporation-dtcc-4464375176</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>Are you ready to make an impact at DTCC? Do you want to work on innovative projects, collaborate with a dynamic and supportive team, and receive investment in your professional development? At DTCC, we are at the forefront of innovation in the financial markets. We are committed to helping our employees grow and succeed. We believe that you have the skills and drive to make a real impact. We foster a thriving internal community and are committed to creating a workplace that looks like the world that we serve. The Information Technology group delivers secure, reliable technology solutions that enable DTCC to be the trusted infrastructure of the global capital markets. The team delivers high-quality information through activities that include development of essential, building infrastructure capabilities to meet client needs and implementing data standards and governance. Pay And Benefits Competitive compensation, including base pay and annual incentive Comprehensive health and life insurance and well-being benefits, based on location Pension / Retirement benefits Paid Time Off and Personal/Family Care, and other leaves of absence when needed to support your physical, financial, and emotional well-being. DTCC offers a flexible/hybrid model of 3 days onsite and 2 days remote (onsite Tuesdays, Wednesdays and a third day unique to each team or employee). The Impact You Will Have In This Role The Development family is responsible for creating, designing, deploying, and supporting applications, programs, and software solutions. May include research, new development, prototyping, modification, reuse, re-engineering, maintenance, or any other activities related to software products used internally or externally on product platforms supported by the firm. The software development process requires in-depth subject matter expertise in existing and emerging development methodologies, tools, and programming languages. Software Developers work closely with business partners and / or external clients in defining requirements and implementing solutions. The Software Development Engineer In Test (SDET) role encompasses automation development and execution, functional, and non-functional testing. The SDET role specializes in the design, development, execution, and maintenance of automated tests to ensure the quality of software products. Partners with team members to understand software requirements and execute automated tests that validate the functionality while considering privacy and security requirements Your Primary Responsibilities Apply different software development and testing methodologies, tools, and technologies Develop, execute, and maintain automated tests across the delivery lifecycle Maintain traceability from user stories through test cases to automated scripts Identify dependencies for environmental and data requirements. Develop applications and construct unit test cases that ensure compliance with functional requirements Follow design and code standards, contributing to continuous improvement discussions Align risk and control processes into day-to day responsibilities to monitor and mitigate risk; escalates appropriately Create and maintain system documentation Support senior team members to implement solutions using software delivery best practices Work with peers to mature ways of working, contributing to continuous testing within the software delivery processes and integrate automated test with CI/CD pipeline Partner with team members to understand software requirements and design automated tests that validate the functionality Collaborate with internal and external teams on development, testing, troubleshooting, and improve overall software quality Aligns risk and control processes into day to day responsibilities to monitor and mitigate risk; escalates appropriately Qualifications Minimum of 4 years of related experience Bachelor's degree preferred or equivalent experience Talents Needed For Success Proven experience leading end-to-end test planning and execution in Agile delivery environments Strong experience in functional testing, automation testing, integration testing, and defect lifecycle management Hands-on experience with test design techniques such as equivalence partitioning, boundary value analysis, decision table testing, pairwise testing, and exploratory testing Experience working with JIRA and ALM/AQM for requirements traceability, test management, reporting, and issue tracking Experience with one or more programming/scripting languages such as Java or Python Experience with automation and API testing tools/frameworks such as Selenium, TestNG, Karate, Rest Assured, or similar Experience with source control and CI/CD tooling such as Git / Bitbucket and Jenkins Familiarity with AI Prompt Engineering, AI Agents, and productivity tooling to improve test design, coverage, and execution efficiency Strong experience validating file-based and data-intensive workflows involving XML, CSV, schema validation, field mappings, transformations, and database verification Experience in financial services, regulatory/reporting processes, onboarding flows, portal-based applications, or data-platform testing preferred Experience coordinating across multiple teams, managing dependencies, and communicating quality status to stakeholders and leadership preferred Actual salary is determined based on the role, location, individual experience, skills, and other considerations. We are an equal opportunity employer and value diversity at our company. We do not discriminate on the basis of race, religion, color, national origin, sex, gender, gender expression, sexual orientation, age, marital status, veteran status, or disability status. We will ensure that individuals with disabilities are provided reasonable accommodation to participate in the job application or interview process, to perform essential job functions, and to receive other benefits and privileges of employment. Please contact us to request accommodation.</t>
         </is>
@@ -1530,21 +1417,21 @@
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Sr Test Engineer - Automation</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/sr-test-engineer-automation-at-clean-harbors-4427621182</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
         <is>
           <t>Clean Harbors</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E24" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -1560,12 +1447,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/sr-test-engineer-automation-at-clean-harbors-4427621182</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
+      <c r="H24" s="3" t="inlineStr">
         <is>
           <t>About CleanHarbors Clean Harbors Inc. (www.cleanharbors.com) is a NYSE listed US based $6.5 billion company. Clean Harbors was founded in 1980 near Boston by Mr. Alan S. McKim . Everywhere industry meets environment, Clean Harbors is on-site, providing premier environmental, energy and industrial services. Clean Harbors employs a dedicated workforce of 25,000 employees and has over 450 service locations across the U.S., Canada and Mexico. Beyond addressing the environmental needs of its more than 300,000 customers, the Company has been on the front lines of addressing some of the largest emergency response events in North America of the past several decades including the BP Oil Spill in the Gulf of Mexico, the anthrax attacks in New York, the 2015 avian flu outbreak that devastated the poultry industry, Hurricanes Katrina, Rita and Sandy, and the oil pipeline breaks that affected the Yellowstone and Kalamazoo rivers, along with other major chemical releases into the environment. Clean Harbors India has been strategically established as the Global Capability Center (GCC) to serve our parent company. We take pride in serving some of the most tech savvy business stakeholders at Clean Harbors. The GCC employees form part of our globally integrated teams that provide cutting-edge IT solutions and production support across platforms. Our shared services teams work seamlessly with their global counterparts in providing critical 24x7 support in various functions including Finance, HR, Procurement, IT and Operations. Our aggressive growth plans open significant career advancement opportunities for our employees. Title: Sr Test Engineer Exp: 5 to 10 Years Location: Hyderabad Working hours: 12.00pm to 9.00pm Education: Bachelors/ Masters degree in computer science or Software Engineering Responsibilities Experience in programming languages like Python, Java, or JavaScript is essential for writing and maintaining automated test scripts Good understanding of QA processes and the software development lifecycle (SDLC) including Agile and DevOps practices Develop Automation scripts for applications developed in .NET framework and full Microsoft stack and SQL Server back end using Selenium tool, create automated scripts, develop functions, add control flow logic, loops etc. for web applications and services Ability to work with and troubleshoot GUI object recognition issues and customize Solid understanding of Object-Oriented programming, design and troubleshooting Participating in preparation of Quality assessments, reports, and metrics formulating go-no go statement based on reports and metrics, test progress and defect status Able to use Pipelines for Test Executions using any of the DevOps tools Identify, analyze, and troubleshoot problems with Automated Test Case runs Stay up to date with emerging trends and technologies in automation testing Work with QA Engineers to identify test scenarios, data requirements, functionality, and areas of application and system level risk Able to effectively work and communicate with local/India and US teams of QA Engineers and Development Team Leads Support in delivering Automation Test plan &amp; Test Strategy for respective Platforms Qualifications 5–10 years of experience in software testing, with at least 3+ years in automation. Strong programming skills in Java, C#. Selenium, Playwright, Cypress, or similar API testing tools like RestAssured, Postman, Karate. Experience in test framework design (BDD/TDD frameworks such as Cucumber, SpecFlow). Familiarity with containerization tools (Docker, Kubernetes). Experience working with microservices architecture. Knowledge of performance testing tools (JMeter, Gatling, etc.). SDET (Software Development Engineer in Test) vs QA-focused role. Specific tech stack (.NET, Java, JavaScript-heavy, etc.) Certifications (ISTQB, Agile Testing) are a plus</t>
         </is>
@@ -1577,21 +1459,21 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>Lead QA Automation Engineer (FX)</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/lead-qa-automation-engineer-fx-at-lseg-4435032613</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
         <is>
           <t>LSEG</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E25" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -1607,12 +1489,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/lead-qa-automation-engineer-fx-at-lseg-4435032613</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr">
         <is>
           <t>Overview: Looking for a QA engineer who strives for a better-quality engineering mindset. As a Senior QA Automation Engineer at LSEG, within our FX vertical, you’ll play a pivotal role in elevating the quality and reliability of advanced FX trading platforms and high-performance, latency-sensitive systems. What Awaits You: Design, develop, and maintain robust automation frameworks using Java, Selenium, Playwright, Cucumber-JVM, SQL, and Maven. Design and execute FIX (Financial Information eXchange) protocol testing across pricing, quote, and order workflows. Perform server-side, API, and integration testing for the PriceStream platform Validate infrastructure and deployments, including infra testing on AWS (Viking) cloud environments. Lead and execute comprehensive QA processes, including functional, regression, API, and database testing. Conduct performance testing (load, stress, fault tolerance). Collaborate closely with cross-functional teams in an Agile environment. Utilize Docker and Kubernetes for test environment setup and automation. Manage multiple projects simultaneously, demonstrating flexibility and adaptability. Champion and implement a shift left approach, embedding quality early in the development lifecycle. Your Winning Qualities: 7+ years of experience in QA automation. Strong knowledge of QA processes and best practices. Hands-on experience with Java, Selenium, Playwright, Cucumber-JVM, SQL, and Maven. Experience with API, GUI, and database testing. Proficient with AI-assisted engineering tools (e.g. GitHub Copilot, Claude Code, Cursor, Codex), and able to drive them to enhance QA and automation productivity. Hands-on experience testing the FIX (Financial Information eXchange) protocol. Strong server-side / backend and integration testing experience. Experience with infrastructure testing and AWS (Viking) cloud environments. Good Understanding of docker and Kubernetes. In-depth understanding of technical architecture, test strategy implementation, and maintaining test plans. Ability to build mocks and simulator components for automation, enabling robust and isolated test environments. What Sets You Apart: Experience with FIX Protocol and Kafka messaging—help us streamline complex trading workflows. Background in FX trading or financial technology—bring your domain expertise to the table. Passion for exploring new tools, frameworks, and testing strategies. A knack for solving tricky performance bottlenecks or debugging distributed systems. Curiosity about financial markets and eagerness to learn beyond your comfort zone. What You’ll Gain: Work with LSEG: Be part of a leading global financial markets infrastructure and data provider, working in our FX vertical at the forefront of financial technology. Hands-On Experience with FX Trading Platforms: Gain in-depth exposure to the world of foreign exchange trading, working on platforms that handle high transaction volumes and require utmost reliability. Exposure to High-Performance, Latency-Intensive Systems: Develop your skills in testing and optimizing systems where speed and performance are critical, preparing you for the most demanding technical challenges in finance. Become a Techno-Functional Expert: This role offers a unique blend of technical and domain knowledge, enabling you to understand both the technology stack and the business logic behind financial products. You’ll become a valuable asset with expertise that bridges the gap between technology and finance. Professional Growth and Learning: Collaborate with industry experts, adopt best practices, and stay updated with the latest tools and technologies in automation, cloud, and financial systems. Ownership and Impact: Enjoy the autonomy to take initiative, drive improvements, and make a tangible impact on the quality and success of mission-critical financial applications. Career Stage: Senior Associate London Stock Exchange Group (LSEG) Information: Join us and be part of a team that values innovation, quality, and continuous improvement. If you're ready to take your career to the next level and make a significant impact, we'd love to hear from you. LSEG is a leading global financial markets infrastructure and data provider. Our purpose is driving financial stability, empowering economies and enabling customers to create sustainable growth. Our purpose is the foundation on which our culture is built. Our values of Integrity, Partnership , Excellence and Change underpin our purpose and set the standard for everything we do, every day. They go to the heart of who we are and guide our decision making and everyday actions. Working with us means that you will be part of a dynamic organisation of 25,000 people across 65 countries. However, we will value your individuality and enable you to bring your true self to work so you can help enrich our diverse workforce. We are proud to be an equal opportunities employer. This means that we do not discriminate on the basis of anyone’s race, religion, colour, national origin, gender, sexual orientation, gender identity, gender expression, age, marital status, veteran status, pregnancy or disability, or any other basis protected under applicable law. Conforming with applicable law, we can reasonably accommodate applicants' and employees' religious practices and beliefs, as well as mental health or physical disability needs. You will be part of a collaborative and creative culture where we encourage new ideas. We are committed to sustainability across our global business and we are proud to partner with our customers to help them meet their sustainability objectives. Our charity, the LSEG Foundation provides charitable grants to community groups that help people access economic opportunities and build a secure future with financial independence. Colleagues can get involved through fundraising and volunteering. LSEG offers a range of tailored benefits and support, including healthcare, retirement planning, paid volunteering days and wellbeing initiatives. Please take a moment to read this privacy notice carefully, as it describes what personal information London Stock Exchange Group (LSEG) (we) may hold about you, what it’s used for, and how it’s obtained, your rights and how to contact us as a data subject. If you are submitting as a Recruitment Agency Partner, it is essential and your responsibility to ensure that candidates applying to LSEG are aware of this privacy notice.</t>
         </is>
@@ -1624,21 +1501,21 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Senior QA Engineer</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/senior-qa-engineer-at-ice-4416491608</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
         <is>
           <t>ICE</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E26" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -1654,12 +1531,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/senior-qa-engineer-at-ice-4416491608</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>Job Purpose The Senior QA Engineer plays a critical role in ensuring the quality, reliability, and performance of the Valuation Analytics application portfolio — including WebAVM, Hoku, and Kokua — by applying advanced QA methodologies and sound judgment to solve complex testing challenges. With a strong foundation in software testing, real estate / AVM domain knowledge, and analytical thinking, this role actively contributes to shaping QA practices across both legacy .NET Framework codebases and modern Angular front-ends. It involves mentoring junior team members, driving process improvements, and fostering a culture of quality throughout the development lifecycle. A proactive mindset and leadership in both technical and collaborative capacities are essential to delivering product excellence in a regulated, data-intensive valuation domain. Responsibilities Assist in leading QA Activities: Plan, design, and execute comprehensive test strategies — including functional, regression, integration, and exploratory testing — across the Valuation Analytics application portfolio. Cover both legacy ASP.NET Web Forms / Web API surfaces and the modern Angular 19 SPA. Perform performance and security testing aligned with organizational standards. Review and Analyze Requirements: Collaborate with Business Analysts, Developers, and End-Users to understand business needs and technical impacts, ensuring test coverage aligns with UAD 3.6, MISMO, and URAR 1004 form requirements, and with downstream partner contracts (Fannie Mae, Chase, Xome). Apply Advanced QA Knowledge: Participate in design reviews to gain a deep understanding of the multi-database architecture (11+ federated SQL Server databases), REST + SOAP integration points, and data workflows. Evaluate requirements for clarity and testability, prioritize high-risk areas — including 800+ UAD validation rules and ML inference paths — contribute to bug triaging to balance quality with delivery timelines, and support release readiness assessments. Develop AI-powered Test Automation Initiatives: Leverage AI-driven tools and techniques to identify and prioritize high-impact test cases for automation. Lead the migration from deprecated Protractor to modern E2E frameworks (Playwright preferred, Cypress, or Selenium 4). Contribute to maintaining code quality and reusability by following established coding standards. Integrate AI-enhanced automation into CI/CD pipelines via Octopus Deploy and Azure DevOps to promote continuous testing across the AVM stack. Problem Solving and Decision Making: Identify, analyze, and provide well-reasoned solutions to complex QA issues — including thread-blocking synchronous code paths, geospatial edge cases, PDF generation timeouts, and combinatorial rule-engine explosion — using established procedures and professional judgement. Recommend improvements to prevent recurrence. Mentorship and Team Development: Guide and train junior QA team members on real estate / AVM domain concepts, test design for federated data sources, and modern automation tooling. Provide feedback and support their professional development. Cross-Team Collaboration: Work closely with Engineering, Data Science, Product, and Operations teams to ensure quality is embedded throughout the development lifecycle for AVM and appraisal workflows. Communicate risks and issues clearly to stakeholders and management. Process Improvement: Contribute to the evaluation and enhancement of QA processes, tools, and metrics across legacy and modern test suites. Wire automated coverage into Octopus Deploy and Azure DevOps pipelines, gate releases on coverage thresholds, and assist in debugging and improving application performance and reliability. System Monitoring and Analysis: Monitor system behavior across DEV / QA / UAT / PRE / PRD / DR environments, analyze trends in valuation throughput, PDF generation pipelines, and ML inference outputs, and proactively identify potential quality issues before they reach production. Knowledge and Experience Bachelor’s degree in accredited institution. 6+ years of experience in software quality assurance, with demonstrated test ownership across both legacy and modern web stacks. Hands-on C# / .NET test authoring — unit and integration tests for ASP.NET Web Forms and Web API codebases (NUnit, Moq, EF6 in-memory). TypeScript / Angular testing — component, service, and observable tests with Jasmine, Karma, TestBed, and HTTP mocking. API testing across REST and SOAP — fluent with both JSON and XML payloads and envelope-aware assertions (Postman, SoapUI, REST Assured, Bruno). SQL Server fluency — query and seed federated databases (KOKUA01, REF01, MLS02, HPT01, DQ02, and 6+ others); strong T-SQL, SSMS, and test-data management. UI automation with modern frameworks — Playwright (preferred), Cypress, or Selenium 4; able to replace deprecated Protractor suites. Hands-on experience writing Python scripts for API testing and data testing — comfortable with data science libraries such as pandas, numpy, scipy, etc. Strong analytical skills and test case design skills; meticulous attention to detail. Solid understanding of the software development life cycle (SDLC) and QA’s role in it. Effective communication and collaboration skills with stakeholders. Strong organizational and time management skills with the ability to work on multiple priorities. Demonstrated ability to solve complex QA problems using sound judgement and existing procedures. Exposure to automation frameworks and scripting languages. Experience using AI tools such as GitHub Copilot, Cursor, or Claude. Preferred Knowledge And Experience Real estate / AVM domain literacy — familiarity with comparables, adjustments, complexity profiles, market trends, URAR 1004, UAD 3.6, MISMO, and MLS data shape. CI/CD pipeline integration — wiring automated suites into Octopus Deploy and Azure DevOps, with coverage gating via ReportPortal or Allure. Document &amp; PDF generation testing — Syncfusion + XSLT pipelines; pixel-diff and structured PDF assertions (pdfplumber, diff-pdf, Applitools). UI automation experience — writing scripts in Playwright (JS), Cypress (JS), and/or Selenium (Java). Familiarity with performance, security, and usability testing. Knowledge of ROI-driven testing strategies. Domain knowledge in finance, mortgage, or real estate.</t>
         </is>
@@ -1671,21 +1543,21 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>V&amp;V Manager</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/v-v-manager-at-cubic-transportation-systems-4436315527</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
         <is>
           <t>Cubic Transportation Systems</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E27" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -1701,12 +1573,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/v-v-manager-at-cubic-transportation-systems-4436315527</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>Business Unit: Cubic Transportation Systems Company Details: When you join Cubic, you become part of a company that creates and delivers technology solutions in transportation to make people’s lives easier by simplifying their daily journeys, and defense capabilities to help promote mission success and safety for those who serve their nation. Led by our talented teams around the world, Cubic is committed to solving global issues through innovation and service to our customers and partners. We have a top-tier portfolio of businesses, including Cubic Transportation Systems (CTS) and Cubic Defense (CD). Explore more on Cubic.com. Job Details: Job Summary: Manage Validation and verification (V&amp;V) activities across complex, multi-disciplinary projects. This role ensures that system-level requirements are thoroughly validated using industry-standard methodologies, automation tools, and collaborative engineering practices. The V&amp;V Principal Engineer plays a critical role in ensuring the quality, performance, and reliability of transit and embedded systems. Key Responsibilities: System-Level V&amp;V Leadership Lead end-to-end validation and verification planning, execution, and reporting. Collaborate with engineering leads to define and trace system requirements to test cases. Drive integration, formal system testing, and procedure validation activities. Team &amp; Resource Management Manage and mentor V&amp;V engineers, overseeing daily activities and performance. Identify test resource needs and manage V&amp;V schedules and budgets. Test Strategy &amp; Execution Develop and maintain V&amp;V plans, test cases, procedures, and reports. Validate software builds and perform test administration. Maintain and enhance the System Test Environment (STE). Automation &amp; Tools Design and implement automated test suites using: Playwright Selenium Cypress Robot Framework RestAssured Postman PyTest Katalon Studio TestNG Perform API testing and SQL-based data validation. Utilize tools such as TestRail, JIRA, Git, Jenkins, and scripting languages for test management and execution. Integrate automation into CI/CD pipelines. Stakeholder Engagement Interface with hardware, software, and systems engineering teams to evaluate test alternatives. Lead Test Readiness Reviews and present V&amp;V status to internal and external stakeholders. Manage and resolve system-level ARQs and issues. Continuous Improvement Stay updated on industry best practices in V&amp;V and test automation. Evaluate vendor capabilities and contribute to procurement decisions. Drive process improvements and standardization across V&amp;V activities. Required Qualifications: Bachelor’s in Technology (B.Tech) or Master’s in Computer Applications (MCA) or related field. Minimum 10+ years of experience in software/system testing, including manual and automated testing. Proven experience in validation and verification of complex engineering or embedded systems. Strong understanding of SDLC, STLC, Agile, and V-model methodologies. Preferred Skills: Experience in Transit domain or Automated Fare Collection Systems (AFCS). Proficiency in Playwright, Selenium, Cypress, API testing, SQL, C++, C#, Java, UNIX, TCP/IP, VB. Hands-on experience with TestRail, JIRA, and test automation frameworks. Excellent communication, leadership, and stakeholder management skills. Generative AI: Exposure to GenAI/ML tools for testing (e.g., GitHub Copilot) BDD: Familiarity with Behavior-Driven Development frameworks like Cucumber Performance Testing: Basic knowledge of performance testing tools such as JMeter ISTQB Foundation level or above. ‎ Worker Type: Employee ‎ We are committed to creating an inclusive workplace and welcome applications from people of all backgrounds. We do not discriminate based on any protected characteristic under applicable law.</t>
         </is>
@@ -1718,21 +1585,21 @@
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Quality Engineer</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/quality-engineer-at-accenture-in-india-4448328660</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
         <is>
           <t>Accenture in India</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E28" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -1748,12 +1615,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/quality-engineer-at-accenture-in-india-4448328660</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>Project Role : Quality Engineer Project Role Description : Enables full stack solutions through multi-disciplinary team planning and ecosystem integration to accelerate delivery and drive quality across the application lifecycle. Performs continuous testing for security, API, and regression suite. Creates automation strategy, automated scripts and supports data and environment configuration. Participates in code reviews, monitors, and reports defects to support continuous improvement activities for the end-to-end testing process. Must have skills : Selenium Good to have skills : NA Minimum 5 Year(s) Of Experience Is Required Educational Qualification : 15 years full time education As a Custom Software Engineer (QE – Automation), you will be responsible for designing, developing, and maintaining robust test automation solutions aligned with business and quality objectives. Your typical day will involve building and enhancing automation frameworks, validating complex systems through UI and API automation, and collaborating closely with cross-functional teams to ensure high-quality, scalable, and reliable software delivery. You will leverage modern automation tools, CI/CD practices, and agile methodologies to improve test efficiency and overall engineering excellence. Roles &amp; Responsibilities: Act as a Subject Matter Expert (SME) for test automation and collaborate with the team to drive high performance and quality outcomes. Take ownership of technical and team-level decisions related to automation strategy, framework enhancements, and tooling. Engage with multiple teams (development, product, DevOps) and contribute to key technical and quality decisions. Design and implement end-to-end automation solutions for UI, API, and database validation. Provide effective solutions to complex testing and automation challenges across the immediate team and multiple teams. Ensure adherence to best practices in automation, coding standards, version control, and CI/CD integration. Facilitate knowledge-sharing sessions, code reviews, and technical discussions to enhance team capability and maturity. Mentor and guide junior team members, supporting their technical growth and career development. Professional &amp; Technical Skills: Must To Have Skills: Strong proficiency in Java-based Selenium automation frameworks, including Cucumber (BDD). Hands-on experience in API and Web Services Automation (REST-based services). Solid experience with Git / Bitbucket for version control and collaborative development. Practical exposure to test and work management tools such as JIRA, Horizon, and Octane. Good working knowledge of Oracle DB and SQL for data validation and backend testing. Secondary / Good To Have Skills: Exposure to Playwright for modern UI automation. Experience or basic working knowledge of RPA tools such as UI Path. Additional Technical Expectations: Strong understanding of test automation frameworks, design patterns, and methodologies. Experience working in CI/CD pipelines and integrating automation with build and deployment processes. Ability to analyze application behavior, debug automation failures, and troubleshoot complex issues effectively. Additional Information: All listed skills should have a minimum of 6+ years of hands-on experience. Overall experience should be 6+ years in Selenium-based automation testing. This position is based at our Chennai/Hyderabad/Bangalore/Coimbatore office. A 15 years of full-time education is mandatory.</t>
         </is>
@@ -1765,21 +1627,21 @@
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>Senior Automation Engineer</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/senior-automation-engineer-at-qualizeal-4471886010</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
         <is>
           <t>QualiZeal</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E29" t="inlineStr">
         <is>
           <t>Mid-Senior level</t>
@@ -1795,12 +1657,7 @@
           <t>193 applicants</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/senior-automation-engineer-at-qualizeal-4471886010</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr">
         <is>
           <t>Position: Senior Automation Test Engineer Location: Hyderabad Experience: 5+Yrs Role Overview: As a Senior Test Engineer , you will be responsible for designing, implementing, and maintaining automated systems. Your role will be critical to enhancing and upholding highest standards of efficiency, quality, and reliability of high-impact systems and applications of our industry-leading clients including Fortune 500 enterprises. You will work on various mission-critical automation projects and collaborate with cross-functional teams to integrate automation technologies successfully across the organization. Job Responsibilities: Testing &amp; Execution: Develop test plans to ensure automated systems meet performance, safety, and functionality standards. Execute automated tests, validate results, and make necessary adjustments to improve the systems. Provide ongoing support and maintenance for automation systems, ensuring minimal downtime. Troubleshoot and resolve issues with automation systems to maintain system reliability. Automation Frameworks: Develop and implement automation scripts for testing across various frameworks and technologies. Deep expertise in Java and Selenium Understanding of integrations with multiple tools across the testing ecosystem. Collaboration &amp; Communication: Collaboration with cross-functional teams for smooth integration of automation technologies. Engage in client interactions to understand requirements and provide updates on testing progress. Why QualiZeal? Award-Winning Workplace : Certified as a Great Place to Work® and recognized by ET NOW as the Best Organization for Women in 2025. Proven Engagement: Industry-recognized client and employee Net Promoter Scores (NPS). Growth-Focused Culture : Equal-opportunity employer with a strong emphasis on leadership development, training, and continuous learning. Flexible &amp; Supportive Environment : We value empathy, recognize contributions, and support work-life balance. Transparent Leadership : Open-book management with a collaborative, inclusive approach. Rapid Growth : 850+ professionals strong and on track to reach 3000+ employees — an exciting time to join. About QualiZeal: QualiZeal is North America's fastest-growing independent digital quality engineering services company. With a diverse portfolio of digital transformation services encompassing Quality Engineering, Digital Engineering, Advisory and Transformation, and Emerging Technology Testing, QualiZeal empowers organizations of all sizes globally to achieve quality excellence and sustainable market leadership. Trusted by 70+ global enterprises and with a headcount of 850+ elite software quality engineers, QualiZeal is pioneering AI-enabled Quality Engineering innovation. QualiZeal has consistently maintained an outstanding client Net Promoter Score (NPS) of over 75, reflecting its unwavering commitment to client satisfaction and service excellence.</t>
         </is>
@@ -1812,21 +1669,21 @@
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>Adv Engineer QE II</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/adv-engineer-qe-ii-at-invesco-4426379205</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
         <is>
           <t>Invesco</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E30" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -1842,12 +1699,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/adv-engineer-qe-ii-at-invesco-4426379205</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
+      <c r="H30" s="3" t="inlineStr">
         <is>
           <t>As one of the world’s leading independent global investment firms, Invesco is dedicated to rethinking possibilities for our clients. By delivering the combined power of our distinctive investment management capabilities, we provide a wide range of investment strategies and vehicles to our clients around the world. If you're looking for challenging work, intelligent colleagues, and exposure across a global footprint, come explore your potential at Invesco. Job Description Key Responsibilities Test Strategy &amp; Planning Develop comprehensive test strategies, test plans, and test cases for complex features and systems. Lead risk assessments to identify critical testing areas and define appropriate testing depth. Participate in requirements analysis, design reviews, and sprint planning to ensure testability and clarity. Test Execution &amp; Automation Execute functional, regression, integration, performance, and security tests. Design and maintain automated test frameworks using industry‑standard tools (e.g., Selenium, Cypress, Playwright, Postman, JMeter). Develop automated test scripts for UI, API, and backend services. Ensure CI/CD pipelines integrate automated test suites effectively. Quality Governance &amp; Process Improvement Establish and improve quality standards, metrics, and best practices. Perform root‑cause analysis for defects and collaborate with engineering to implement long‑term fixes. Drive continuous improvement in development and testing processes using Agile, Scrum, or DevOps methodologies. Contribute to scaling testing capabilities across teams through tools, training, and documentation. Cross‑Functional Collaboration Partners with developers to ensure early detection and resolution of issues. Work closely with product owners to validate acceptance criteria and ensure high‑quality user experiences. Mentor junior SQA analysts on testing best practices, tools, and automation techniques. Communicate test progress, risks, and results to stakeholders in a clear and actionable manner. Qualifications Education &amp; Experience Bachelor’s degree in Computer Science, Software Engineering, Information Systems, or related technical field. 4–7+ years of experience in software quality assurance or test engineering. Demonstrated experience with test automation frameworks and scripting languages (Python, JavaScript, Java, etc.). Experience testing in Agile/Scrum environments. Technical Skills Strong understanding of software QA methodologies, tools, and processes. Experience with test automation tools such as Selenium, Cypress, Playwright, Appium, or similar. Proficiency in API testing tools (Postman, SoapUI, REST‑Assured). Familiarity with CI/CD systems (Azure DevOps, Jenkins, GitHub Actions, GitLab CI, etc.). Solid grasp of SQL, NoSQL, and data validation techniques. Experience with cloud platforms (Azure, AWS, GCP) is a plus. Soft Skills Strong analytical and problem‑solving abilities. Excellent communication skills and the ability to work in cross‑functional teams. Detail‑oriented with strong organizational and documentation skills. Ability to mentor others and influence quality culture across teams. Preferred Certifications ISTQB (Foundation or Advanced Level) Certified Software Quality Analyst (CSQA) Agile or Scrum certification DevOps or Cloud certifications (AWS/Azure/GCP) Full Time / Part Time Full time Worker Type Employee Job Exempt (Yes / No) No Workplace Model At Invesco, our workplace model supports our culture and meets the needs of our clients while providing flexibility our employees value. As a full-time employee, compliance with the workplace policy means working with your direct manager to create a schedule where you will work in your designated office at least three days a week, with two days working outside an Invesco office. Why Invesco In Invesco, we act with integrity and do meaningful work to create impact for our stakeholders. We believe our culture is stronger when we all feel we belong, and we respect each other’s identities, lives, health, and well-being. We come together to create better solutions for our clients, our business and each other by building on different voices and perspectives. We nurture and encourage each other to ensure our meaningful growth, both personally and professionally. We believe in diverse, inclusive, and supportive workplace where everyone feels equally valued, and this starts at the top with our senior leaders having diversity and inclusion goals. Our global focus on diversity and inclusion has grown exponentially and we encourage connection and community through our many employee-led Business Resource Groups (BRGs). What’s in it for you? As an organization we support personal needs, diverse backgrounds and provide internal networks, as well as opportunities to get involved in the community and in the world. Our benefit policy includes but not limited to: Competitive Compensation Flexible, Hybrid Work 30 days’ Annual Leave + Public Holidays Life Insurance Retirement Planning Group Personal Accident Insurance Medical Insurance for Employee and Family Annual Health Check-up 26 weeks Maternity Leave Paternal Leave Adoption Leave Near site Childcare Facility Employee Assistance Program Study Support Employee Stock Purchase Plan ESG Commitments and Goals Business Resource Groups Career Development Programs Mentoring Programs Invesco Cares Dress for your Day In Invesco, we offer development opportunities that help you thrive as a lifelong learner in a constantly evolving business environment and ensure your constant growth. Our AI enabled learning platform delivers curated content based on your role and interest. We ensure our manager and leaders also have many opportunities to advance their skills and competencies that becomes pivotal in their continuous pursuit of performance excellence. To Know More About Us About Invesco: https://www.invesco.com/corporate/en/home.html About our Culture: https://www.invesco.com/corporate/en/about-us/our-culture.html About our D&amp;I policy: https://www.invesco.com/corporate/en/our-commitments/diversity-and-inclusion.html About our CR program: https://www.invesco.com/corporate/en/our-commitments/corporate-responsibility.html Apply for the role @ Invesco Careers : https://careers.invesco.com/india/</t>
         </is>
@@ -1859,21 +1711,21 @@
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>Senior Quality Engineer (Automation -  Selenium, Playwright, Cypress)</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/senior-quality-engineer-automation-selenium-playwright-cypress-at-s-p-global-4470707634</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
         <is>
           <t>S&amp;P Global</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E31" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -1889,12 +1741,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/senior-quality-engineer-automation-selenium-playwright-cypress-at-s-p-global-4470707634</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr">
         <is>
           <t>About The Role: Grade Level (for internal use): 09 S&amp;P Global Dow Jones Indices The Role: Senior Quality Engineer About The Role: Senior Quality Engineer with extensive experience in test automation, API validation, data quality assurance, and enterprise application testing. Proven expertise in designing scalable automation frameworks, validating complex business workflows, and supporting CI/CD delivery pipelines. Experienced in Agentic AI testing, including validation of autonomous agents, multi-agent orchestration workflows, tool invocation testing, and identification of edge cases unique to AI-driven systems. Strong background in financial services, data validation, Agile methodologies, and quality engineering best practices. The Team: The S&amp;P Dow Jones Indices Technology Quality Engineering team comprises of global teams that are responsible for the quality and delivery of applications and infrastructure that power global markets. What’s In It For You: This role provides great opportunities for career growth and professional development. You will build new skills, share knowledge, participate in innovative solutions and work on the latest technologies. Be part of S&amp;P Dow Jones Indices providers of iconic and innovative index solutions, bringing transparency to global capital markets. In addition, you will be part of a Global inclusive team where creativity, collaboration and open-mindedness are valued. Key Responsibilities Quality Engineering &amp; Automation Design, develop, and maintain automated test frameworks for web applications and APIs. Create and execute comprehensive test plans, test cases, and regression suites. Perform functional, integration, regression, and end-to-end testing across multiple platforms. Validate backend services, APIs, and database integrations to ensure data accuracy and system reliability. Collaborate with Product Managers, Developers, Business Analysts, and other stakeholders to ensure requirements are testable and quality standards are met. Analyse defects, perform root cause analysis, and track issues through resolution using tools such as Jira or Azure DevOps. Support CI/CD pipelines by integrating automated tests into continuous delivery workflows. Participate in release validation, deployment verification, and production support activities Technical Skills Test Automation: Playwright, Selenium, Cypress, TestNG, Junit Programming Languages: Python, Java, JavaScript, TypeScript API Testing: Postman, REST APIs, API Automation Database Testing: SQL, Data Validation DevOps &amp; Tools: Git, Azure DevOps, Jira, Jenkins, CI/CD Pipelines AI &amp; Agentic Systems: Agentic AI, Multi-Agent Systems, Workflow Validation, Autonomous Testing Qualifications: Bachelor's degree in computer science, Information Systems or Engineering is required, or in lieu, a demonstrated equivalence in work experience 4+ years of experience in complete software testing activities Knowledge of Agentic AI concepts, autonomous systems, and multi-agent orchestration frameworks. Experience working with AI-powered applications, LLMs, chatbots, or intelligent automation platforms. Experience testing REST APIs using Postman, Swagger, or automated API testing frameworks. Familiarity with AI evaluation, prompt testing, observability, and model validation techniques. Experience with CI/CD tools such as GitHub Actions, Azure DevOps Pipelines, Jenkins, or GitLab. Exposure to cloud platforms such as AWS, Azure, or Google Cloud. Experience in performance, security, or reliability testing. Strong SQL skills for data validation and database testing. Domain experience in Financial Services, Capital Markets, Asset Management, or Data Analytics is a plus. Experience with Index/Benchmarks and Asset Management is a plus Experience and understanding of Agile methodology Excellent analytical and problem-solving skills, with a keen attention to detail Strong communication and interpersonal skills, with the ability to effectively collaborate with cross-functional teams About Company Statement: S&amp;P Global delivers essential intelligence that powers decision making. We provide the world’s leading organizations with the right data, connected technologies and expertise they need to move ahead. As part of our team, you’ll help solve complex challenges that equip businesses, governments and individuals with the knowledge to adapt to a changing economic landscape. S&amp;P Dow Jones Indices provides iconic and innovative index solutions, bringing transparency to global capital markets. About S&amp;P Global Dow Jones Indices At S&amp;P Dow Jones Indices, we provide iconic and innovative index solutions backed by unparalleled expertise across the asset-class spectrum. By bringing transparency to the global capital markets, we empower investors everywhere to make decisions with conviction. We’re the largest global resource for index-based concepts, data and research, and home to iconic financial market indicators, such as the S&amp;P 500® and the Dow Jones Industrial Average®. More assets are invested in products based upon our indices than any other index provider in the world. With over USD 7.4 trillion in passively managed assets linked to our indices and over USD 11.3 trillion benchmarked to our indices, our solutions are widely considered indispensable in tracking market performance, evaluating portfolios and developing investment strategies. S&amp;P Dow Jones Indices is a division of S&amp;P Global (NYSE: SPGI). S&amp;P Global is the world’s foremost provider of credit ratings, benchmarks, analytics and workflow solutions in the global capital, commodity and automotive markets. With every one of our offerings, we help many of the world’s leading organizations navigate the economic landscape so they can plan for tomorrow, today. For more information, visit www.spglobal.com/spdji. What’s In It For You? Our Mission: Advancing Essential Intelligence. Our People: We're more than 35,000 strong worldwide—so we're able to understand nuances while having a broad perspective. Our team is driven by curiosity and a shared belief that Essential Intelligence can help build a more prosperous future for us all.From finding new ways to measure sustainability to analyzing energy transition across the supply chain to building workflow solutions that make it easy to tap into insight and apply it. We are changing the way people see things and empowering them to make an impact on the world we live in. We’re committed to a more equitable future and to helping our customers find new, sustainable ways of doing business. Join us and help create the critical insights that truly make a difference. Our Values: Integrity, Discovery, Partnership Throughout our history, the world's leading organizations have relied on us for the Essential Intelligence they need to make confident decisions about the road ahead. We start with a foundation of integrity in all we do, bring a spirit of discovery to our work, and collaborate in close partnership with each other and our customers to achieve shared goals. Benefits: We take care of you, so you can take care of business. We care about our people. That’s why we provide everything you—and your career—need to thrive at S&amp;P Global. Our Benefits Include: Health &amp; Wellness: Health care coverage designed for the mind and body. Flexible Downtime: Generous time off helps keep you energized for your time on. Continuous Learning: Access a wealth of resources to grow your career and learn valuable new skills. Invest in Your Future: Secure your financial future through competitive pay, retirement planning, a continuing education program with a company-matched student loan contribution, and financial wellness programs. Family Friendly Perks: It’s not just about you. S&amp;P Global has perks for your partners and little ones, too, with some best-in class benefits for families. Beyond the Basics: From retail discounts to referral incentive awards—small perks can make a big difference. For more information on benefits by country visit: https://spgbenefits.com/benefit-summaries Global Hiring And Opportunity At S&amp;P Global: At S&amp;P Global, we are committed to fostering a connected and engaged workplace where all individuals have access to opportunities based on their skills, experience, and contributions. Our hiring practices emphasize fairness, transparency, and merit, ensuring that we attract and retain top talent. By valuing different perspectives and promoting a culture of respect and collaboration, we drive innovation and power global markets. Recruitment Fraud Alert: If you receive an email from a spglobalind.com domain or any other regionally based domains, it is a scam and should be reported to reportfraud@spglobal.com. S&amp;P Global never requires any candidate to pay money for job applications, interviews, offer letters, “pre-employment training” or for equipment/delivery of equipment. Stay informed and protect yourself from recruitment fraud by reviewing our guidelines, fraudulent domains, and how to report suspicious activity here. Equal Opportunity Employer S&amp;P Global is an equal opportunity employer and all qualified candidates will receive consideration for employment without regard to race/ethnicity, color, religion, sex, sexual orientation, gender identity, national origin, age, disability, marital status, military veteran status, unemployment status, or any other status protected by law. Only electronic job submissions will be considered for employment. If you need an accommodation during the application process due to a disability, please send an email to: EEO.Compliance@spglobal.com and your request will be forwarded to the appropriate person. US Candidates Only: The EEO is the Law Poster http://www.dol.gov/ofccp/regs/compliance/posters/pdf/eeopost.pdf describes discrimination protections under federal law. Pay Transparency Nondiscrimination Provision - https://www.dol.gov/sites/dolgov/files/ofccp/pdf/pay-transp_%20English_formattedESQA508c.pdf 20 - Professional (EEO-2 Job Categories-United States of America), IFTECH202.1 - Middle Professional Tier I (EEO Job Group) Job ID: 330894 Posted On: 2026-09-25 Location: Hyderabad, Telangāna, India</t>
         </is>
@@ -1906,21 +1753,21 @@
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Quality Engineer [T500-29719]</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/quality-engineer-t500-29719-at-cibc-india-4472002175</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
         <is>
           <t>CIBC India</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E32" t="inlineStr">
         <is>
           <t>Mid-Senior level</t>
@@ -1936,12 +1783,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/quality-engineer-t500-29719-at-cibc-india-4472002175</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
+      <c r="H32" s="3" t="inlineStr">
         <is>
           <t>About CIBC: CIBC is a leading North American bank, with a history of more than 150 years of living our purpose - to help make your ambition a reality. Client relationships are at the center of our strategy, and our growth is enabled by a highly engaged and connected global team. From digital banking to community impact, we’re proud to drive progress for our clients and our communities. Recognized for our culture, award-winning innovation and community investment, CIBC continues to evolve by putting people and progress at the centre of everything we do. About CIBC India: CIBC India is a technology and operations hub in Hyderabad, where you’ll be part of our highly engaged and global team, and play a central role in supporting our growth. Whether you’re driving innovation in digital banking or streamlining client onboarding, you’ll be part of a culture recognized for excellence and investment in people. At CIBC India, people and progress are at the center of what we do: you’ll develop skills, collaborate with industry leaders, and see your ideas realized in a culture that values progress and belonging. We provide cutting-edge resources, ongoing learning, and a supportive environment where people come first. If you’re ready to create meaningful change and build your future, CIBC India is where your ambition meets opportunity. What CIBC India Offers: At CIBC India, your goals are a priority. We start with your strengths and ambitions and strive to create opportunities to tap into your potential. We aspire to give you a career that goes well beyond your compensation. We work to recognize you in meaningful, personalized ways including competitive fixed pay, performance-based incentive programs, a family-first benefits program, employer contributions for your retirement, attractive time off and leave offerings, wellbeing support, and MomentMakers, our social, points-based recognition program. Our spaces and technological toolkit will make it simple to bring together great minds to create innovative solutions that make a difference for our clients worldwide We cultivate a culture where you can express your ambition through initiatives like Purpose Day, a paid day off dedicated for you to use to invest in your growth and development. What You’ll Be Doing (position summary): The Quality Engineer is responsible for developing and executing manual and automated test scenarios and scripts for system integration and acceptance testing of banking platforms, in compliance with established controls and standards. The role collaborates with development teams to ensure quality deliverables, analyzes test results, and provides actionable insights to stakeholders. The Quality Engineer also contributes to process improvement initiatives and maintains quality metrics, supporting the continuous improvement of testing practices within the organization. At CIBC India we enable the work environment most optimal for you to thrive in your role. Details on your work arrangement (including on-site and remote work) will be discussed at the time of your interview. How You’ll Succeed (responsibilities): Testing Expertise: Participate in requirements and design reviews to provide feedback from a quality perspective. Develop and maintain test suites (manual/automated) and create test scripts using scripting languages. Execute test cases, document test results, raise defects, and collaborate with development teams for resolution. Analyze test results and provide actionable insights to stakeholders. Contribute to process improvement initiatives and quality metrics reporting. Leadership Skills: Provide advice to team members, support, and mentorship. Proactively identify potential issues throughout all test phases and suggest improvements or enhancements. Project Coordination: Identify obstacles or risks that may impact a project’s timeline or success and provide regular status updates. Ensure all test deliverables are received, approved, and aligned to project timelines, budgets, and goals. Maintain strong attention to detail and organizational skills. CROSS-FUNCTIONAL RELATIONSHIPS: Collaborates with software developers to build automated solutions and resolve defects. Works closely with business stakeholders and technology partners to ensure testing requirements are understood and met. Communicates with project managers and other cross-functional teams to provide updates and escalate issues as needed. As an employee of CIBC, the incumbent must comply with all applicable CIBC and Line of Business policies, standards, guidelines and controls. As a key contributor to the business unit, this job has the authority to recommend changes to business processes in order to enhance operational efficiency and effectiveness. JOB DIMENSIONS: Scope includes testing for multiple banking platforms and projects. Responsible for supporting quality assurance across various geographies and business lines as assigned. Provides advisory and support services to project teams and stakeholders to ensure quality standards are met. Experience: 3+ years of experience. Who You Are (skills/qualifications): Must Have Skills: 3+ years of experience in a Quality Engineering or equivalent technical role, preferably within the banking sector. Database knowledge - RDBMS (Relational Database Management Systems)/Source-to-Target Mapping (STM)/ ETL testing SQL scripting expertise - Ability to write medium to complex SQL queries Working knowledge of cloud/Azure environment (e.g., Databricks) Experience in preparing test plans and test cases &amp; responsible for execution Strong analytical and problem-solving skills. Effective communication skills to convey technical concepts to non-technical audiences. Collaboration and teamwork skills. Continuous learning mindset to stay updated with emerging technologies and regulatory developments. Good knowledge of QE Processes, Testing Life Cycle, SDLC, and Defect Management processes. Good to Have: Defect and Test management tools (Any tool - JIRA/OpenText ALM/Confluence) Automation Testing (Any tools - Tosca DI/Selenium/Robot Framework/Parasoft SOAtest/Postman/RestAssured/ Cucumber) Unix knowledge - For running and initiating jobs in UAT/SIT environments Identify Test Data requirements Hands-on experience with test automation tools (e.g., Tosca DI, Selenium, Robot framework, Parasoft SOAtest, Postman, RestAssured, Cucumber) for testing REST and Web Services. Preferred experience with Python, Java Understanding of debugging and analyzing code logs and development techniques. Experience with test management tools (e.g., JIRA, HP ALM). Privacy: By proceeding with the creation of a profile and submitting an application in response to this job posting, you acknowledge and agree that your personal data will be collected, used, retained and disclosed by CIBC India and its affiliates, as described in the Candidate Privacy Statement.</t>
         </is>
@@ -1953,21 +1795,21 @@
           <t>2026-09-25</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>Sr. Software QA Automation Engineer</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/sr-software-qa-automation-engineer-at-revvity-4444760646</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
         <is>
           <t>Revvity</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E33" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -1983,12 +1825,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/sr-software-qa-automation-engineer-at-revvity-4444760646</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr">
         <is>
           <t>Role Purpose Assist in designing test plans and writing/executing test cases for functional and/or performance testing within the assigned domain, leveraging Playwright with TypeScript for automation. Work as a member of the scrum team, including planning, estimating, and verifying user stories and acceptance criteria. Develop strong expertise in the assigned domain areas. Design and implement automated test scripts using Playwright with TypeScript. Effectively communicate status, metrics, and issues on a regular basis. Understand and comply with Revvity Signals practices. Assist in creating high-quality test summary reports with well-structured written content. Become a user expert on how our products work, understanding strengths and weaknesses, and advocating for customer issues to enhance their experience. Create and execute integrated automated test cases with Playwright, working in conjunction with manual testers and manual test cases. Job Specifications Qualifications Computer Science and/or Science-based bachelor’s degree 7+ years of experience qualifying high-volume, scalable enterprise software Excellent experience working in an agile/scrum environment Excellent working knowledge of Windows/Linux operating systems Excellent understanding of Quality Assurance life cycle, methodologies, and best practices Excellent knowledge in test case management and bug tracking systems such as Jira, Zephyr Minimum 5 years of experience with one of the automation tools like Playwright, TestComplete, Selenium is necessary Experience with databases and data platforms Experience testing systems at a large scale is a plus Experience with developing API test frameworks Experience with Playwright and Selenium for UI automation Excellent experience in transforming manual test cases into automated test cases Experience in test documentation, defect analysis, tracking, and reporting Java, .NET, or TypeScript development experience required Special Skills &amp; Knowledge Solid experience in the domain assigned to Good English, written and verbal Key Competencies Passion for quality Ability to respectfully speak up on quality matters Strong emphasis on good UI design with meticulous attention to detail Self-motivated, independent thinker with excellent troubleshooting skills Ability to learn quickly and stay current with new technologies Ability to work within a multi-site, multicultural team</t>
         </is>
@@ -2000,21 +1837,21 @@
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>SDET II [T500-29659]</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/sdet-ii-t500-29659-at-marriott-tech-accelerator-4471458809</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
         <is>
           <t>Marriott Tech Accelerator</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E34" t="inlineStr">
         <is>
           <t>Mid-Senior level</t>
@@ -2030,12 +1867,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/sdet-ii-t500-29659-at-marriott-tech-accelerator-4471458809</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
+      <c r="H34" s="3" t="inlineStr">
         <is>
           <t>About Us: Marriott International Inc. , headquartered in Bethesda, Maryland, USA, was founded in May 1927 by J. Willard Marriott and Alice S. Marriott with a modest nine-seat A&amp;W root beer stand. Guided by the family's leadership and core principles, Marriott International today has grown into a global hospitality giant, operating approximately 10,000 properties and over 30 leading brands in more than 140 countries and territories. From such humble beginnings to becoming the world’s largest hotel company, Marriott International has never stopped searching for inventive ways to serve its customers, provide opportunities for its associates, and grow their business. At Marriott Tech Accelerator center (MTA), Hyderabad, India, Marriott is exploring the world we live in and all its possibilities. At Marriott Tech Accelerator, we are a team of passionate engineering minds dedicated to creating and building cutting-edge solutions that streamline operations and elevate guest experiences. Marriott Tech Accelerator is an ANSR entity incorporated exclusively for providing services to Marriott International. Role Title: SDET II Position Summary: We are looking for a highly skilled and detail-oriented SDET to join our quality engineering team. This role requires strong experience in test automation, microservices testing, and enterprise platforms such as Salesforce. The ideal candidate will also have hands-on expertise with tools like Playwright and Postman, and a passion for delivering high-quality, scalable software solutions. Candidate will work across multiple products &amp; engineering teams to deliver incremental value against Loyalty Platform roadmap. Perform research, analysis, design, creation, and implementation of applications to meet current and future user requirements. Help develop proof-of-concept implementations to help evaluate cutting-edge technology to drive and meet Marriott business &amp; technology objectives. Candidate must have the ability to communicate upward to superiors and laterally to other departments. Job Responsibilities: Design and implement automated test frameworks for Salesforce applications, including UI, API, and end-to-end testing. Develop and execute automated tests for microservices-based architectures, ensuring reliability, scalability, and performance. Utilize Playwright for model-based test automation, including test case design, execution, and maintenance. Perform API testing using Postman, validating service contracts, data flows, and integration points. Collaborate with developers, product owners, and QA analysts to define test strategies and ensure comprehensive coverage. Integrate automated tests into CI/CD pipelines using tools like Jenkins, GitHub Actions, or Azure DevOps. Monitor test execution, analyze failures, and provide actionable feedback to development teams. Participate in Agile ceremonies and contribute to sprint planning, retrospectives, and continuous improvement initiatives Skill and Experience: 7 + years of experience in software testing and automation. Hands-on experience with Salesforce testing, including declarative and programmatic components will be a big plus Good understanding of microservices architecture and testing strategies for distributed systems. Experience with Postman for API testing and automation. Proficient in leveraging Postman for API testing, validation, and automation. Strong programming skills in languages such as Java, Python, or JavaScript for developing and maintaining automation frameworks. Hands-on experience with leading test automation frameworks and tools, including Selenium, Playwright, Cypress, TestNG, and JMeter, with proficiency in at least one modern automation platform such as Selenium or Playwright, along with test data management solutions Ability to design, implement, and maintain scalable automated testing solutions across UI, API, and performance testing domains. Experience with version control systems (e.g., Git) and CI/CD tools. Bachelor’s degree in computer science, Engineering, or related field, or equivalent experience. Strong analytical skills, attention to detail, and a passion for quality. Education and Certifications: Undergraduate degree in Computer Science or related technical field or equivalent experience/certification Work location: Hyderabad, India. Work mode: Hybrid Marriott’s core values: At Marriott, our core values make us who we are. We believe that success is never final. As we change and grow, the beliefs that are most important to us stay the same—putting people first, pursuing excellence, embracing change, acting with integrity, and serving our world. Being part of Marriott Tech Accelerator means being part of a proud history and a thriving culture</t>
         </is>
@@ -2047,21 +1879,21 @@
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>Automation Engineer with Playwright</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/automation-engineer-with-playwright-at-algoleap-4471457186</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
         <is>
           <t>algoleap</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E35" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -2077,12 +1909,7 @@
           <t>129 applicants</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/automation-engineer-with-playwright-at-algoleap-4471457186</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr">
         <is>
           <t>We are looking for a highly skilled and detail-oriented Senior QA Automation Engineer with strong expertise in Playwright, Java Selenium, Java Cucumber, and modern test automation practices. The ideal candidate will be responsible for designing scalable automation frameworks, developing automated test suites, validating APIs and backend systems, and ensuring high-quality software releases through continuous testing within CI/CD pipelines. This role requires close collaboration with Product Owners, Developers, Business Analysts, and DevOps teams in an Agile environment. Key Responsibilities Â· Design, Develop, And Maintain Robust Automation Frameworks Using Playwright (JavaScript/TypeScript) Selenium WebDriver with Java Cucumber BDD Framework Â· Create And Execute Automated Test Scripts For Functional Testing Regression Testing End-to-End Testing Smoke and Sanity Testing Cross-browser Testing Â· Integrate automation suites into CI/CD pipelines using Azure DevOps and support release validation activities. Â· Develop and maintain reusable automation components, utilities, and libraries to improve test efficiency and scalability. Â· Perform API testing using tools such as Postman, REST Assured, or equivalent technologies. Â· Validate backend data through SQL queries and database testing. Â· Analyze application requirements, user stories, and acceptance criteria to create comprehensive test scenarios and test cases. Â· Identify defects, perform root cause analysis, track issues, and collaborate with development teams for timely resolution. Â· Review automation code and enforce testing best practices, naming standards, and framework guidelines. Â· Monitor automation execution results, maintain test metrics, and generate quality reports for stakeholders. Â· Participate actively in Agile Scrum ceremonies including Sprint Planning, Daily Standups, Backlog Refinement, Sprint Reviews, and Retrospectives. Â· Mentor junior QA engineers and contribute to continuous improvement initiatives within the QA organization. Â· Support performance, security, and accessibility testing initiatives when required. Required Technical Skills Automation Testing Â· Playwright (JavaScript/TypeScript) – Advanced Â· Selenium WebDriver with Java Â· Cucumber BDD Framework Â· TestNG / JUnit Programming Languages Â· Java Â· JavaScript / TypeScript API Testing Â· REST API Testing Â· Postman Â· REST Assured Â· JSON/XML validation CI/CD &amp; DevOps Â· Azure DevOps Pipelines Â· Git / GitHub / Azure Repos Â· Continuous Testing Practices Database Testing Â· SQL Â· Data Validation and Reconciliation Â· Query Optimization and Troubleshooting Agile Tools Â· Azure DevOps Boards Â· Jira Â· Confluence</t>
         </is>
@@ -2094,21 +1921,21 @@
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>QA Automation Engineer – Playwright</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/qa-automation-engineer-%E2%80%93-playwright-at-algoleap-4471449740</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
         <is>
           <t>algoleap</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E36" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -2124,12 +1951,7 @@
           <t>168 applicants</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/qa-automation-engineer-%E2%80%93-playwright-at-algoleap-4471449740</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
+      <c r="H36" s="3" t="inlineStr">
         <is>
           <t>We are looking for a highly skilled and detail-oriented Senior QA Automation Engineer with strong expertise in Playwright, Java Selenium, Java Cucumber, and modern test automation practices. The ideal candidate will be responsible for designing scalable automation frameworks, developing automated test suites, validating APIs and backend systems, and ensuring high-quality software releases through continuous testing within CI/CD pipelines. This role requires close collaboration with Product Owners, Developers, Business Analysts, and DevOps teams in an Agile environment. Key Responsibilities Â· Design, Develop, And Maintain Robust Automation Frameworks Using Playwright (JavaScript/TypeScript) Selenium WebDriver with Java Cucumber BDD Framework Â· Create And Execute Automated Test Scripts For Functional Testing Regression Testing End-to-End Testing Smoke and Sanity Testing Cross-browser Testing Â· Integrate automation suites into CI/CD pipelines using Azure DevOps and support release validation activities. Â· Develop and maintain reusable automation components, utilities, and libraries to improve test efficiency and scalability. Â· Perform API testing using tools such as Postman, REST Assured, or equivalent technologies. Â· Validate backend data through SQL queries and database testing. Â· Analyze application requirements, user stories, and acceptance criteria to create comprehensive test scenarios and test cases. Â· Identify defects, perform root cause analysis, track issues, and collaborate with development teams for timely resolution. Â· Review automation code and enforce testing best practices, naming standards, and framework guidelines. Â· Monitor automation execution results, maintain test metrics, and generate quality reports for stakeholders. Â· Participate actively in Agile Scrum ceremonies including Sprint Planning, Daily Standups, Backlog Refinement, Sprint Reviews, and Retrospectives. Â· Mentor junior QA engineers and contribute to continuous improvement initiatives within the QA organization. Â· Support performance, security, and accessibility testing initiatives when required. Required Technical Skills Automation Testing Â· Playwright (JavaScript/TypeScript) – Advanced Â· Selenium WebDriver with Java Â· Cucumber BDD Framework Â· TestNG / JUnit Programming Languages Â· Java Â· JavaScript / TypeScript API Testing Â· REST API Testing Â· Postman Â· REST Assured Â· JSON/XML validation CI/CD &amp; DevOps Â· Azure DevOps Pipelines Â· Git / GitHub / Azure Repos Â· Continuous Testing Practices Database Testing Â· SQL Â· Data Validation and Reconciliation Â· Query Optimization and Troubleshooting Agile Tools Â· Azure DevOps Boards Â· Jira Â· Confluence Preferred Qualifications Â· Experience implementing Playwright automation from scratch. Â· Experience working in cloud environments such as Azure or AWS. Â· Knowledge of Docker, containerized testing, and modern DevOps practices. Â· Familiarity with performance testing tools such as JMeter. Â· Experience testing enterprise applications, web portals, APIs, and reporting platforms. Â· Understanding of test automation design patterns and framework architecture. Â· Exposure to Power BI, Grafana, or analytics/reporting platforms is a plus. Soft Skills Â· Strong analytical and problem-solving abilities. Â· Excellent communication and stakeholder management skills. Â· Ability to work independently and drive quality initiatives. Â· Strong collaboration and mentoring capabilities. Â· Proactive mindset with focus on continuous improvement. Â· Ability to handle multiple projects and deadlines in a fast-paced Agile environment. Education Â· Bachelor's or Master's degree in Computer Science, Information Technology, Engineering, or related field. Nice to Have Â· Playwright with TypeScript. Â· Contract/API Mocking experience. Â· Visual testing automation. Â· Accessibility testing knowledge. Â· Experience with test reporting tools such as Allure, Extent Reports, or ReportPortal. Â· AI-assisted testing tools and test automation accelerators. Experience Required: 7–12 Years Primary Skill: Playwright Automation (JavaScript/TypeScript) Secondary Skills: Java, Selenium, Cucumber, Azure DevOps, API Testing, SQL, Agile Scrum.</t>
         </is>
@@ -2141,21 +1963,21 @@
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>Senior Software Engineer - Quality</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/senior-software-engineer-quality-at-agilent-technologies-4469238239</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
         <is>
           <t>Agilent Technologies</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E37" t="inlineStr">
         <is>
           <t>Mid-Senior level</t>
@@ -2171,12 +1993,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/senior-software-engineer-quality-at-agilent-technologies-4469238239</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr">
         <is>
           <t>Job Description We are seeking a highly skilled and experienced Senior Software Engineer QA to help deliver high-quality digital experiences across Agilent.com and its connected applications. In this role, you will design and implement scalable automated testing solutions, validate critical product and content experiences, and partner closely with development, product, content, and centralized testing teams to improve release quality, reliability, and speed. You will play a key role in strengthening QA coverage across functional, regression, integration, content functional quality validation, and performance testing while mentoring others and promoting modern quality engineering practices. This role currently follows a hybrid work model. Work arrangements may evolve based on future business needs. What you’ll do: Work with a team of engineers to deliver feature set that are crucial to Revenue growth. Be a part of a world class global organization. Automate test cases as part of each sprint to support in-sprint testing, faster validation, and higher release confidence. Design and develop comprehensive automation test scripts and frameworks for our constantly updating A/B testing and personalization workflows. Collaborate with centralized testing team to integrate automated tests into the CI/CD pipeline. Collaborate with the development team to understand product features and technical specifications to create effective test plans and strategies. Perform functional, regression, and performance testing. Analyze test results, identify defects, and work with developers to resolve them. Mentor QA engineers to deliver better QA coverage and results. Qualifications Required: Bachelor’s or master’s Degree or equivalent. 6+ years of relevant experience in QA and automation dev. Hands-on experience with Playwright for full end-to-end automation, including test design, execution, debugging, and maintenance across modern web applications. Collaborate with the development team to understand product features and technical specifications to create effective test plans and strategies. Perform functional, regression, and performance testing. Analyze test results, identify defects, and work with developers to resolve them. Experience writing exceptional test cases in JIRA, Cucumber etc. Experience with test automation frameworks like Selenium, Cypress, Playwright, or Appium. Solid understanding of the AI-assisted software development lifecycle (SDLC) and QA methodologies. Experience with setting up test automation with CI/CD tools (e.g., Jenkins, GitLab CI). Experience with GitHub Actions for CI/CD is a must. Programming skills in Python, JavaScript, React, Java Excellent problem-solving skills and attention to detail. Strong communication skills and a collaborative perspective. Experience in Using generative AI for test case generation and execution Ways to stand out: Ability to fully utilize agentic development techniques, including AI-assisted coding, automated test generation, code review support, documentation acceleration, and workflow automation, to improve engineering efficiency, delivery speed, and overall development quality. QA automation for testing in the eCommerce domain. Test automation integration with CI/CD. Additional Details This job has a full time weekly schedule. Our pay ranges are determined by role, level, and location. Within the range, individual pay is determined by work location and additional factors, including job-related skills, experience, and relevant education or training. During the hiring process, a recruiter can share more about the specific pay range for a preferred location. Pay and benefit information by country are available at: https://careers.agilent.com/locations Agilent Technologies Inc. is an equal opportunity employer. Qualified applicants will receive consideration for employment without regard to race, color, religion, sex, sexual orientation, gender identity, national origin, protected veteran status, disability or any other protected categories under all applicable laws. Travel Required: Occasional Shift: Day Duration: No End Date Job Function: IT</t>
         </is>
@@ -2188,21 +2005,21 @@
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>Lead QA Engineer</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/lead-qa-engineer-at-healthedge-4435135055</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
         <is>
           <t>HealthEdge</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Greater Hyderabad Area</t>
-        </is>
-      </c>
       <c r="E38" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -2218,12 +2035,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/lead-qa-engineer-at-healthedge-4435135055</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
+      <c r="H38" s="3" t="inlineStr">
         <is>
           <t>Overview JOB DESCRIPTION QUALITY ENGINEERING QA Automation Lead Test Automation Framework Architect | Playwright + TypeScript About The Role We are looking for a hands-on QA Automation Lead to drive test automation strategy and execution across the GuidingCare ® platform. You will design, architect, and evolve scalable automation frameworks using Playwright (TypeScript) and Selenium, lead our framework modernization, mentor a strong team of automation engineers, and partner with development to embed in-sprint automation as a default. Key Responsibilities Framework &amp; Architecture Design, build, and maintain scalable automation frameworks from scratch using Playwright with TypeScript Lead modernization of legacy suites ( Katalon , Selenium) to Playwright-based frameworks Establish design patterns (POM), reusable libraries, utilities, and reporting plug-ins for cross-team adoption Define and ma in tain automation coding standards, branching strategy, and code review practices Strategy &amp; Execution Define automation strategy, coverage targets, and KPIs aligned with release and business goals Lead in-sprint automation — partner with dev teams to comple te the automation alongside features . improve regression suite pass rates through systematic flaky-test triage and root-cause analysis Integrate test automation deeply into CI/CD pipelines ( A WS , GitHub Actions) Leadership &amp; Mentorship Mentor and coach QA engineers on automation and framework usage Lead by example — write production-grade automation code that others use as the reference AI-Assisted Testing Champion the use of AI tooling (Copilot, Claude, Playwright Test Generator) to accelerate authoring, maintenance, and adoption of emerging AI/ML approaches in testing Reporting &amp; Stakeholder Management Develop execution reports and dashboards to track progress, test outcomes, and quality metrics, providing clear visibility to leadership stakeholders Partner with Product, Dev, and DevOps to embed quality earlier in the SDLC Required Skills Must-Have 1 0 + years of overall QA / SDET experience, with 8 + years in test automation Deep expertise in Playwright with TypeScript — test architecture, fixtures, parallelization, network interception, visual testing, debugging Strong hands-on experience with Selenium WebDriver (Java or JavaScript bindings) Proven track record of building automation frameworks from scratch . Strong programming skill s in TypeScript / JavaScript , P ytho n , Java . API automation experience (Playwright API testing, REST Assured, Postman) CI/CD integration experience — AW S preferred; GitHub Actions also acceptable Proficient with Git, pull-request workflows, and modern development practices Strong analytical and root-cause debugging skills, with excellent written and verbal communication Nice-to-Have Domain experience in healthcare . Performance testing experience . Cloud platform experience (AWS) Hands-on with AI-assisted testing tools . Exposure to accessibility testing and open-source contributions to automation projects Experience with test management tools (Zephyr Essential, TestRail) Experience in developing accessibility test automation solutions using AI-driven tools and frameworks Education Bachelor’s or master’s degree in computer science , Engineering, or a related field</t>
         </is>
@@ -2235,21 +2047,21 @@
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>Senior Associate, Quality Assurance Engineer, Regional Wealth Delivery</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/senior-associate-quality-assurance-engineer-regional-wealth-delivery-at-dbs-bank-4443373266</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
         <is>
           <t>DBS Bank</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Greater Hyderabad Area</t>
-        </is>
-      </c>
       <c r="E39" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -2265,12 +2077,7 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/senior-associate-quality-assurance-engineer-regional-wealth-delivery-at-dbs-bank-4443373266</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr">
         <is>
           <t>Business Function Group Technology and Operations (T&amp;O) enables and empowers the bank with an efficient, nimble and resilient infrastructure through a strategic focus on productivity, quality &amp; control, technology, people capability and innovation. In Group T&amp;O, we manage the majority of the Bank's operational processes and inspire to delight our business partners through our multiple banking delivery channels.. Roles &amp; Responsibilities As a QA Engineer you should have working knowledge on Git. (Anything apart from BitBucket are good to have). You should know how to view quality holistically and ensure the highest software quality. At least 5 years of relevant experience in testing mobile (Android, iOS) applications using automated test scripts. Experience in API testing and automation frameworks. Should know how to work with Jira, Jenkins, Docker, etc. Solid coding background in Java, Objective-C, JavaScript or similar with at least 3yrs of experience. Experience with at least one of the following technologies: Cucumber, Appium, Selenium, XCode UI Automation, Espresso, (mobile testing tools and frameworks). Experience with basic UNIX commands and working knowledge on LINUX flavor. Hands-on experience tool like and SOAP UI, REST API. Requirements A graduate in computers or Engineering from a reputed university. 10+ years’ experience in Mobile testing. Should have strong analytic skills to process complex requirement to come up with end to end scenarios and test cases Hands on experience in Agile projects Banking experience is preferred Location: Hyderabad - DTI Waverock SEZ Job: Technology Schedule: Regular Employee Status: Full time</t>
         </is>
@@ -2282,21 +2089,21 @@
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>IN_Senior Associate_.Net Fullstack Developer_GCC_Advisory_Hyderabad</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/in-senior-associate-net-fullstack-developer-gcc-advisory-hyderabad-at-pwc-india-4471638566</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
         <is>
           <t>PwC India</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Greater Hyderabad Area</t>
-        </is>
-      </c>
       <c r="E40" t="inlineStr">
         <is>
           <t>Mid-Senior level</t>
@@ -2312,12 +2119,7 @@
           <t>Be among the first 25 applicants</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/in-senior-associate-net-fullstack-developer-gcc-advisory-hyderabad-at-pwc-india-4471638566</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
+      <c r="H40" s="3" t="inlineStr">
         <is>
           <t>Line of Service Advisory Industry/Sector Not Applicable Specialism Operations Management Level Senior Associate Job Description &amp; Summary At PwC, our people in business application consulting specialise in consulting services for a variety of business applications, helping clients optimise operational efficiency. These individuals analyse client needs, implement software solutions, and provide training and support for seamless integration and utilisation of business applications, enabling clients to achieve their strategic objectives. As a business application consulting generalist at PwC, you will provide consulting services for a wide range of business applications. You will leverage a broad understanding of various software solutions to assist clients in optimising operational efficiency through analysis, implementation, training, and support. * Why PWC At PwC , you will be part of a vibrant community of solvers that leads with trust and creates distinctive outcomes for our clients and communities. This purpose-led and values-driven work, powered by technology in an environment that drives innovation, will enable you to make a tangible impact in the real world. We reward your contributions, support your wellbeing, and offer inclusive benefits, flexibility programmes and mentorship that will help you thrive in work and life. Together, we grow, learn, care, collaborate, and create a future of infinite experiences for each other. Learn more about us .At PwC , we believe in providing equal employment opportunities, without any discrimination on the grounds of gender, ethnic background, age, disability, marital status, sexual orientation, pregnancy, gender identity or expression, religion or other beliefs, perceived differences and status protected by law. We strive to create an environment where each one of our people can bring their true selves and contribute to their personal growth and the firm’s growth. To enable this, we have zero tolerance for any discrimination and harassment based on the above considerations. " Job Description &amp; Summary: We are looking for a seasoned Automation Engineer Responsibilities: Expertise in Selenium with any programming language (Cypress, Java, Python, C#, Java script) Mandatory skill sets: - Logical programming and debugging skills. - Automation framework development/enhancement experience is a must. - Experience in robot framework is a plus. - Experience in a fast-paced agile environment. - Good interpersonal and communication skills - Good debugging skills and an ability to identify issues quickly and effectively - Experience in developing automation framework for testing Restful web services - Experience in Jenkins, configuring jobs, executing TestNG test cases from Jenkins - Good Understanding about Data structure and algorithms - Good knowledge on Relational Database/SQL Queries - Worked on Manual functional/regression/integration testing - Strong understanding of APIs and experience of automating APIs Preferred skill sets: Cypress, Java, Python, C#, Java script technologies such as Docker, Kubernetes, and OpenShift. ·  Provide input on improving the development process and software performance across the team. Years of experience required: 4 to 9 years Education qualification: BE/ B.Tech /MBA /MCA Education (if blank, degree and/or field of study not specified) Degrees/Field of Study required: Bachelor of Engineering, MBA (Master of Business Administration) Degrees/Field of Study preferred: Certifications (if blank, certifications not specified) Required Skills QA Automation Optional Skills Accepting Feedback, Accepting Feedback, Active Listening, AI Fluency, AI-Human Collaboration, Analytical Reasoning, Analytical Thinking, Application Software, Business Data Analytics, Business Management, Business Technology, Business Transformation, Communication, Creativity, Digital Tooling, Documentation Development, Embracing Change, Emotional Regulation, Empathy, Implementation Research, Implementation Support, Implementing Technology, Inclusion, Intellectual Curiosity, Learning Agility {+ 19 more} Desired Languages (If blank, desired languages not specified) Travel Requirements Not Specified Available for Work Visa Sponsorship? No Government Clearance Required? No Job Posting End Date June 30, 2026</t>
         </is>
@@ -2329,21 +2131,21 @@
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>Guidewire QA Lead</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/guidewire-qa-lead-at-valuemomentum-4469665980</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
         <is>
           <t>ValueMomentum</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E41" t="inlineStr">
         <is>
           <t>Not Applicable</t>
@@ -2359,12 +2161,7 @@
           <t>56 applicants</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/guidewire-qa-lead-at-valuemomentum-4469665980</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
+      <c r="H41" s="3" t="inlineStr">
         <is>
           <t>Job Title: Guidewire QA Lead Job ID: POS-20674 Primary Skill: Guidewire Key Skills: Guidewire ClaimCenter QA, Playwright Automation, BDD with Cucumber, Cypress, GT UI, GT API, P&amp;C Insurance Mode of Work: Work From Office Job Location: Hyderabad / Pune Experience: 8+ Years About The Job We are seeking a highly skilled and experienced Quality Engineer Lead to join our dynamic team. The ideal candidate will have experience developing and implementing testing automation frameworks, with strong expertise in both UI and API-based testing automation and automation strategies for unit testing. Know your team At ValueMomentum’s Engineering Center, we are a team of passionate engineers who thrive on tackling complex business challenges with innovative solutions while transforming the P&amp;C insurance value chain. We achieve this through a strong engineering foundation and continuously refining our processes, methodologies, tools, agile delivery teams and core engineering archetypes. Our core expertise lies in Cloud Engineering, Application Engineering, Data Engineering, Core Engineering, Quality Engineering and Domain expertise. Join a team that invests in your growth. Our Infinity Program empowers you to build your career with role-specific skill development leveraging immersive learning platforms. You'll have the opportunity to showcase your talents by contributing to impactful projects. Responsibilities Lead and manage testing efforts for Guidewire ClaimCenter, integrations and forms testing. Lead and mentor a team of quality engineers to ensure high standards of quality and performance. Develop, maintain and execute automated test scripts using Playwright, Selenium with Java, Cypress, GT UI and GT API. Implement and manage BDD frameworks using Cucumber. Develop comprehensive test plans covering functional test design and execution approaches. Develop test cases based on business requirements and system specifications. Execute test cases and scenarios to ensure thorough testing coverage. Conduct functional testing to ensure software meets business requirements and specifications. Identify, document and track defects and issues through resolution. Collaborate with business analysts, developers, product managers and other stakeholders to understand system requirements and ensure accurate testing. Review team members’ test cases and deliverables and ensure compliance with industry standards and best practices in P&amp;C insurance and Guidewire. Utilize Agile methodologies to drive efficient testing processes and deliver high-quality software solutions. Identify and escalate issues and risks and work with project managers and stakeholders toward timely resolution. Continuously improve testing processes and strategies to enhance quality and efficiency. Stay updated on industry trends and best practices in Guidewire ClaimCenter, PolicyCenter, BillingCenter and P&amp;C insurance. Track team status and share daily, weekly and monthly status reports with client stakeholders. Requirements Bachelor’s degree in Computer Science, Information Technology or a related field. Minimum 8 years of experience in quality engineering and automation testing. Proficiency in Playwright, Selenium with Java, Cypress, GT UI, GT API and BDD with Cucumber. Strong understanding of functional testing principles and practices. Experience in P&amp;C Insurance, Claims and Guidewire ClaimCenter. Excellent leadership and team management skills. Strong analytical and problem-solving abilities. Excellent communication and interpersonal skills. Good To Have Experience with other automation tools and frameworks. Knowledge of CI/CD pipelines. Familiarity with Agile and Scrum methodologies. About The Company Founded in 2000 with the core belief that impactful change comes from deep commitment, ValueMomentum specializes in delivering measurable results across the P&amp;C value stream. For more than 25 years, we have empowered more than 100 carriers to reimagine their businesses with AI and emerging technologies, navigate market shifts, unlock speed to value, and become future-ready. We help insurers in the US, Canada, and Europe stay ahead with sustained growth and high performance to enhance stakeholder value and foster resilient societies. Our culture – Our fuel At ValueMomentum, we believe in making employees win by nurturing them from within, collaborating and looking out for each other. People firs - Empower employees to succeed. Nurture leaders - Nurture from within. Enjoy wins - Recognize and celebrate win. Collaboration - Foster a culture of collaboration and people-centricity. Diversity - Committed to diversity, equity, and inclusion. Fun - Create a fun and engaging work environment Company Benefits Compensation - Competitive compensation package comparable to the best in the industry. Career Growth - Career development, comprehensive training &amp; certification programs, and fast track growth for high potential associates. Health Benefits: Comprehensive health benefits and life insurance.</t>
         </is>
@@ -2376,21 +2173,21 @@
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>Test Engineer</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>https://in.linkedin.com/jobs/view/test-engineer-at-tata-consultancy-services-4469393691</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
         <is>
           <t>Tata Consultancy Services</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Hyderabad, Telangana, India</t>
-        </is>
-      </c>
       <c r="E42" t="inlineStr">
         <is>
           <t>Mid-Senior level</t>
@@ -2406,61 +2203,97 @@
           <t>Over 200 applicants</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>https://in.linkedin.com/jobs/view/test-engineer-at-tata-consultancy-services-4469393691</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
+      <c r="H42" s="3" t="inlineStr">
         <is>
           <t>Location: HYDERABAD Experience Range: 5- 8 Yrs MUST SKILLS: Automation Testing with Selenium, Java Job Description SOAPUI, Python, Java, Selenium Exposure in creating Cucumber reports Automation Testing Frameworks like TestNG, JUnit, Pytest Understanding of REST APIs, MicroServices Good communication skills and ability to work independently with the different teams. .</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I42"/>
+  <autoFilter ref="A1:H42"/>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId82"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>